<commit_message>
test results 1st record, pdf template
</commit_message>
<xml_diff>
--- a/web-console/server/assets/pdf_template.xlsx
+++ b/web-console/server/assets/pdf_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\DEV\UBA6\web-console\server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{195F4861-F82F-4AFB-B39A-1D35FCC8B078}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52BDB272-97B4-47CF-A21C-0C4D96146F4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
   <si>
     <t>Wh</t>
   </si>
@@ -93,32 +93,6 @@
   </si>
   <si>
     <t>UBA6 Report</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">[הערה: הכנסת </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>כל</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> שלבי  הניסוי, עם תוצאות]</t>
-    </r>
   </si>
   <si>
     <t>Current [mA]</t>
@@ -236,7 +210,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -302,42 +276,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color theme="0" tint="-0.24994659260841701"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="0" tint="-0.24994659260841701"/>
-      </top>
-      <bottom style="thin">
-        <color theme="0" tint="-0.24994659260841701"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="0" tint="-0.24994659260841701"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
@@ -359,14 +304,10 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -378,8 +319,8 @@
     <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5822,8 +5763,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="614350" y="401783"/>
-          <a:ext cx="9325165" cy="4265799"/>
+          <a:off x="609732" y="402938"/>
+          <a:ext cx="9277828" cy="4213844"/>
           <a:chOff x="614350" y="401783"/>
           <a:chExt cx="9325165" cy="4265799"/>
         </a:xfrm>
@@ -6294,7 +6235,7 @@
     <col min="4" max="9" width="19.6640625" style="2" customWidth="1"/>
     <col min="10" max="10" width="9.44140625" style="2" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="4.109375" style="2" customWidth="1"/>
-    <col min="12" max="12" width="9.109375" style="18"/>
+    <col min="12" max="12" width="9.109375" style="15"/>
     <col min="13" max="13" width="82.44140625" style="2" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="123.33203125" style="2" customWidth="1"/>
     <col min="15" max="15" width="78.88671875" style="2" customWidth="1"/>
@@ -6302,7 +6243,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="J1" s="19"/>
+      <c r="J1" s="16"/>
     </row>
     <row r="2" spans="2:14" ht="8.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="3"/>
@@ -6323,7 +6264,7 @@
       </c>
       <c r="E3" s="8"/>
       <c r="F3" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H3" s="7" t="s">
         <v>1</v>
@@ -6349,266 +6290,266 @@
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B5" s="12"/>
-      <c r="C5" s="22"/>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="18"/>
+      <c r="I5" s="18"/>
+      <c r="J5" s="18"/>
       <c r="K5" s="13"/>
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B6" s="12"/>
-      <c r="C6" s="22"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="22"/>
-      <c r="J6" s="22"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
       <c r="K6" s="13"/>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B7" s="12"/>
-      <c r="C7" s="22"/>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="22"/>
-      <c r="I7" s="22"/>
-      <c r="J7" s="22"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="18"/>
       <c r="K7" s="13"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B8" s="12"/>
-      <c r="C8" s="22"/>
-      <c r="D8" s="22"/>
-      <c r="E8" s="22"/>
-      <c r="F8" s="22"/>
-      <c r="G8" s="22"/>
-      <c r="H8" s="22"/>
-      <c r="I8" s="22"/>
-      <c r="J8" s="22"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="18"/>
       <c r="K8" s="13"/>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B9" s="12"/>
-      <c r="C9" s="22"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="22"/>
-      <c r="F9" s="22"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="22"/>
-      <c r="I9" s="22"/>
-      <c r="J9" s="22"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="18"/>
+      <c r="H9" s="18"/>
+      <c r="I9" s="18"/>
+      <c r="J9" s="18"/>
       <c r="K9" s="13"/>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B10" s="12"/>
-      <c r="C10" s="22"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="22"/>
-      <c r="F10" s="22"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="22"/>
-      <c r="I10" s="22"/>
-      <c r="J10" s="22"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18"/>
+      <c r="H10" s="18"/>
+      <c r="I10" s="18"/>
+      <c r="J10" s="18"/>
       <c r="K10" s="13"/>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B11" s="12"/>
-      <c r="C11" s="22"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
-      <c r="G11" s="22"/>
-      <c r="H11" s="22"/>
-      <c r="I11" s="22"/>
-      <c r="J11" s="22"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="18"/>
+      <c r="I11" s="18"/>
+      <c r="J11" s="18"/>
       <c r="K11" s="13"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B12" s="12"/>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
-      <c r="G12" s="22"/>
-      <c r="H12" s="22"/>
-      <c r="I12" s="22"/>
-      <c r="J12" s="22"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="18"/>
+      <c r="I12" s="18"/>
+      <c r="J12" s="18"/>
       <c r="K12" s="13"/>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B13" s="12"/>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
-      <c r="G13" s="22"/>
-      <c r="H13" s="22"/>
-      <c r="I13" s="22"/>
-      <c r="J13" s="22"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="18"/>
+      <c r="G13" s="18"/>
+      <c r="H13" s="18"/>
+      <c r="I13" s="18"/>
+      <c r="J13" s="18"/>
       <c r="K13" s="13"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B14" s="12"/>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
-      <c r="G14" s="22"/>
-      <c r="H14" s="22"/>
-      <c r="I14" s="22"/>
-      <c r="J14" s="22"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="18"/>
+      <c r="H14" s="18"/>
+      <c r="I14" s="18"/>
+      <c r="J14" s="18"/>
       <c r="K14" s="13"/>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B15" s="12"/>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="22"/>
-      <c r="I15" s="22"/>
-      <c r="J15" s="22"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="18"/>
+      <c r="I15" s="18"/>
+      <c r="J15" s="18"/>
       <c r="K15" s="13"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B16" s="12"/>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="22"/>
-      <c r="H16" s="22"/>
-      <c r="I16" s="22"/>
-      <c r="J16" s="22"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="18"/>
+      <c r="H16" s="18"/>
+      <c r="I16" s="18"/>
+      <c r="J16" s="18"/>
       <c r="K16" s="13"/>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B17" s="12"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="22"/>
-      <c r="H17" s="22"/>
-      <c r="I17" s="22"/>
-      <c r="J17" s="22"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18"/>
+      <c r="F17" s="18"/>
+      <c r="G17" s="18"/>
+      <c r="H17" s="18"/>
+      <c r="I17" s="18"/>
+      <c r="J17" s="18"/>
       <c r="K17" s="13"/>
     </row>
     <row r="18" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B18" s="12"/>
-      <c r="C18" s="22"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="22"/>
-      <c r="I18" s="22"/>
-      <c r="J18" s="22"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="18"/>
+      <c r="J18" s="18"/>
       <c r="K18" s="13"/>
     </row>
     <row r="19" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B19" s="12"/>
-      <c r="C19" s="22"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="22"/>
-      <c r="H19" s="22"/>
-      <c r="I19" s="22"/>
-      <c r="J19" s="22"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="18"/>
+      <c r="G19" s="18"/>
+      <c r="H19" s="18"/>
+      <c r="I19" s="18"/>
+      <c r="J19" s="18"/>
       <c r="K19" s="13"/>
     </row>
     <row r="20" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B20" s="12"/>
-      <c r="C20" s="22"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="22"/>
-      <c r="H20" s="22"/>
-      <c r="I20" s="22"/>
-      <c r="J20" s="22"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="18"/>
+      <c r="F20" s="18"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="18"/>
+      <c r="J20" s="18"/>
       <c r="K20" s="13"/>
     </row>
     <row r="21" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B21" s="12"/>
-      <c r="C21" s="22"/>
-      <c r="D21" s="22"/>
-      <c r="E21" s="22"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="22"/>
-      <c r="H21" s="22"/>
-      <c r="I21" s="22"/>
-      <c r="J21" s="22"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="18"/>
+      <c r="G21" s="18"/>
+      <c r="H21" s="18"/>
+      <c r="I21" s="18"/>
+      <c r="J21" s="18"/>
       <c r="K21" s="13"/>
     </row>
     <row r="22" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B22" s="12"/>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="22"/>
-      <c r="H22" s="22"/>
-      <c r="I22" s="22"/>
-      <c r="J22" s="22"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="18"/>
+      <c r="E22" s="18"/>
+      <c r="F22" s="18"/>
+      <c r="G22" s="18"/>
+      <c r="H22" s="18"/>
+      <c r="I22" s="18"/>
+      <c r="J22" s="18"/>
       <c r="K22" s="13"/>
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B23" s="12"/>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="22"/>
-      <c r="H23" s="22"/>
-      <c r="I23" s="22"/>
-      <c r="J23" s="22"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="18"/>
+      <c r="F23" s="18"/>
+      <c r="G23" s="18"/>
+      <c r="H23" s="18"/>
+      <c r="I23" s="18"/>
+      <c r="J23" s="18"/>
       <c r="K23" s="13"/>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B24" s="12"/>
-      <c r="C24" s="22"/>
-      <c r="D24" s="22"/>
-      <c r="E24" s="22"/>
-      <c r="F24" s="22"/>
-      <c r="G24" s="22"/>
-      <c r="H24" s="22"/>
-      <c r="I24" s="22"/>
-      <c r="J24" s="22"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="18"/>
+      <c r="G24" s="18"/>
+      <c r="H24" s="18"/>
+      <c r="I24" s="18"/>
+      <c r="J24" s="18"/>
       <c r="K24" s="13"/>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B25" s="12"/>
-      <c r="C25" s="22"/>
-      <c r="D25" s="22"/>
-      <c r="E25" s="22"/>
-      <c r="F25" s="22"/>
-      <c r="G25" s="22"/>
-      <c r="H25" s="22"/>
-      <c r="I25" s="22"/>
-      <c r="J25" s="22"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="18"/>
+      <c r="F25" s="18"/>
+      <c r="G25" s="18"/>
+      <c r="H25" s="18"/>
+      <c r="I25" s="18"/>
+      <c r="J25" s="18"/>
       <c r="K25" s="13"/>
     </row>
     <row r="26" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B26" s="12"/>
-      <c r="C26" s="22"/>
-      <c r="D26" s="22"/>
-      <c r="E26" s="22"/>
-      <c r="F26" s="22"/>
-      <c r="G26" s="22"/>
-      <c r="H26" s="22"/>
-      <c r="I26" s="22"/>
-      <c r="J26" s="22"/>
+      <c r="C26" s="18"/>
+      <c r="D26" s="18"/>
+      <c r="E26" s="18"/>
+      <c r="F26" s="18"/>
+      <c r="G26" s="18"/>
+      <c r="H26" s="18"/>
+      <c r="I26" s="18"/>
+      <c r="J26" s="18"/>
       <c r="K26" s="13"/>
       <c r="M26" s="14"/>
     </row>
@@ -6630,8 +6571,10 @@
       <c r="I28" s="8"/>
       <c r="J28" s="8"/>
       <c r="K28" s="9"/>
-      <c r="L28" s="21"/>
-      <c r="M28" s="15"/>
+      <c r="L28" s="17"/>
+      <c r="M28" s="23"/>
+      <c r="N28" s="23"/>
+      <c r="O28" s="23"/>
     </row>
     <row r="29" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B29" s="12"/>
@@ -6639,24 +6582,26 @@
         <v>13</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
-      <c r="I29" s="23"/>
+      <c r="I29" s="19"/>
       <c r="K29" s="13"/>
-      <c r="L29" s="21"/>
-      <c r="M29" s="16"/>
+      <c r="L29" s="17"/>
+      <c r="M29" s="23"/>
+      <c r="N29" s="23"/>
+      <c r="O29" s="23"/>
     </row>
     <row r="30" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B30" s="12"/>
       <c r="H30" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
-      <c r="I30" s="23"/>
+      <c r="I30" s="19"/>
       <c r="K30" s="13"/>
-      <c r="L30" s="17"/>
-      <c r="M30" s="17"/>
-      <c r="N30" s="17"/>
-      <c r="O30" s="17"/>
+      <c r="L30" s="6"/>
+      <c r="M30" s="22"/>
+      <c r="N30" s="22"/>
+      <c r="O30" s="22"/>
     </row>
     <row r="31" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B31" s="12"/>
@@ -6666,12 +6611,12 @@
       <c r="H31" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="I31" s="23"/>
+      <c r="I31" s="19"/>
       <c r="K31" s="13"/>
-      <c r="L31" s="17"/>
-      <c r="M31" s="17"/>
-      <c r="N31" s="17"/>
-      <c r="O31" s="17"/>
+      <c r="L31" s="6"/>
+      <c r="M31" s="22"/>
+      <c r="N31" s="22"/>
+      <c r="O31" s="22"/>
     </row>
     <row r="32" spans="2:15" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B32" s="6"/>
@@ -6682,59 +6627,59 @@
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
       <c r="H32" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
-      <c r="I32" s="23"/>
+      <c r="I32" s="19"/>
       <c r="J32" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K32" s="9"/>
-      <c r="L32" s="17"/>
-      <c r="M32" s="17"/>
-      <c r="N32" s="17"/>
-      <c r="O32" s="17"/>
+      <c r="L32" s="6"/>
+      <c r="M32" s="22"/>
+      <c r="N32" s="22"/>
+      <c r="O32" s="22"/>
     </row>
     <row r="33" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B33" s="12"/>
       <c r="H33" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
-      <c r="I33" s="23"/>
+      <c r="I33" s="19"/>
       <c r="J33" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="K33" s="13"/>
-      <c r="L33" s="17"/>
-      <c r="M33" s="17"/>
-      <c r="N33" s="17"/>
-      <c r="O33" s="17"/>
+      <c r="L33" s="6"/>
+      <c r="M33" s="22"/>
+      <c r="N33" s="22"/>
+      <c r="O33" s="22"/>
     </row>
     <row r="34" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B34" s="12"/>
       <c r="H34" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="I34" s="23"/>
+      <c r="I34" s="19"/>
       <c r="J34" s="2" t="s">
         <v>1</v>
       </c>
       <c r="K34" s="13"/>
-      <c r="L34" s="17"/>
-      <c r="M34" s="17"/>
-      <c r="N34" s="17"/>
-      <c r="O34" s="17"/>
+      <c r="L34" s="6"/>
+      <c r="M34" s="22"/>
+      <c r="N34" s="22"/>
+      <c r="O34" s="22"/>
     </row>
     <row r="35" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B35" s="12"/>
       <c r="H35" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I35" s="23"/>
+      <c r="I35" s="19"/>
       <c r="K35" s="13"/>
-      <c r="L35" s="17"/>
-      <c r="M35" s="17"/>
-      <c r="N35" s="17"/>
-      <c r="O35" s="17"/>
+      <c r="L35" s="6"/>
+      <c r="M35" s="22"/>
+      <c r="N35" s="22"/>
+      <c r="O35" s="22"/>
     </row>
     <row r="36" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B36" s="12"/>
@@ -6744,12 +6689,12 @@
       <c r="H36" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="I36" s="23"/>
+      <c r="I36" s="19"/>
       <c r="K36" s="13"/>
-      <c r="L36" s="17"/>
-      <c r="M36" s="17"/>
-      <c r="N36" s="17"/>
-      <c r="O36" s="17"/>
+      <c r="L36" s="6"/>
+      <c r="M36" s="22"/>
+      <c r="N36" s="22"/>
+      <c r="O36" s="22"/>
     </row>
     <row r="37" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B37" s="12"/>
@@ -6759,12 +6704,12 @@
       <c r="H37" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="I37" s="23"/>
+      <c r="I37" s="19"/>
       <c r="K37" s="13"/>
-      <c r="L37" s="17"/>
-      <c r="M37" s="17"/>
-      <c r="N37" s="17"/>
-      <c r="O37" s="17"/>
+      <c r="L37" s="6"/>
+      <c r="M37" s="22"/>
+      <c r="N37" s="22"/>
+      <c r="O37" s="22"/>
     </row>
     <row r="38" spans="2:15" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B38" s="6"/>
@@ -6772,35 +6717,33 @@
         <v>3</v>
       </c>
       <c r="K38" s="9"/>
-      <c r="L38" s="17"/>
-      <c r="M38" s="17"/>
-      <c r="N38" s="17"/>
-      <c r="O38" s="17"/>
+      <c r="L38" s="6"/>
+      <c r="M38" s="22"/>
+      <c r="N38" s="22"/>
+      <c r="O38" s="22"/>
     </row>
     <row r="39" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B39" s="12"/>
-      <c r="D39" s="25" t="s">
-        <v>17</v>
-      </c>
-      <c r="E39" s="25"/>
-      <c r="F39" s="25"/>
-      <c r="G39" s="25"/>
-      <c r="H39" s="25"/>
-      <c r="I39" s="25"/>
-      <c r="J39" s="25"/>
+      <c r="D39" s="21"/>
+      <c r="E39" s="21"/>
+      <c r="F39" s="21"/>
+      <c r="G39" s="21"/>
+      <c r="H39" s="21"/>
+      <c r="I39" s="21"/>
+      <c r="J39" s="21"/>
       <c r="K39" s="13"/>
-      <c r="L39" s="17"/>
-      <c r="M39" s="17"/>
-      <c r="N39" s="17"/>
-      <c r="O39" s="17"/>
+      <c r="L39" s="6"/>
+      <c r="M39" s="22"/>
+      <c r="N39" s="22"/>
+      <c r="O39" s="22"/>
     </row>
     <row r="40" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B40" s="12"/>
       <c r="K40" s="13"/>
-      <c r="L40" s="17"/>
-      <c r="M40" s="17"/>
-      <c r="N40" s="17"/>
-      <c r="O40" s="17"/>
+      <c r="L40" s="6"/>
+      <c r="M40" s="22"/>
+      <c r="N40" s="22"/>
+      <c r="O40" s="22"/>
     </row>
     <row r="41" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B41" s="12"/>
@@ -6815,320 +6758,311 @@
       <c r="I41" s="8"/>
       <c r="J41" s="8"/>
       <c r="K41" s="13"/>
-      <c r="L41" s="17"/>
-      <c r="M41" s="17"/>
-      <c r="N41" s="17"/>
-      <c r="O41" s="17"/>
+      <c r="L41" s="6"/>
+      <c r="M41" s="22"/>
+      <c r="N41" s="22"/>
+      <c r="O41" s="22"/>
     </row>
     <row r="42" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B42" s="12"/>
       <c r="K42" s="13"/>
-      <c r="L42" s="17"/>
-      <c r="M42" s="17"/>
-      <c r="N42" s="17"/>
-      <c r="O42" s="17"/>
+      <c r="L42" s="6"/>
+      <c r="M42" s="22"/>
+      <c r="N42" s="22"/>
+      <c r="O42" s="22"/>
     </row>
     <row r="43" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B43" s="12"/>
       <c r="K43" s="13"/>
-      <c r="L43" s="17"/>
-      <c r="M43" s="17"/>
-      <c r="N43" s="17"/>
-      <c r="O43" s="17"/>
+      <c r="L43" s="6"/>
+      <c r="M43" s="22"/>
+      <c r="N43" s="22"/>
+      <c r="O43" s="22"/>
     </row>
     <row r="44" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B44" s="12"/>
       <c r="K44" s="13"/>
-      <c r="L44" s="17"/>
-      <c r="M44" s="17"/>
-      <c r="N44" s="17"/>
-      <c r="O44" s="17"/>
+      <c r="L44" s="6"/>
+      <c r="M44" s="22"/>
+      <c r="N44" s="22"/>
+      <c r="O44" s="22"/>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B45" s="12"/>
       <c r="K45" s="13"/>
-      <c r="L45" s="17"/>
-      <c r="M45" s="17"/>
-      <c r="N45" s="17"/>
-      <c r="O45" s="17"/>
+      <c r="L45" s="6"/>
+      <c r="M45" s="22"/>
+      <c r="N45" s="22"/>
+      <c r="O45" s="22"/>
     </row>
     <row r="46" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="12"/>
       <c r="K46" s="13"/>
-      <c r="L46" s="17"/>
-      <c r="M46" s="17"/>
-      <c r="N46" s="17"/>
-      <c r="O46" s="17"/>
+      <c r="L46" s="6"/>
+      <c r="M46" s="22"/>
+      <c r="N46" s="22"/>
+      <c r="O46" s="22"/>
     </row>
     <row r="47" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="12"/>
       <c r="K47" s="13"/>
-      <c r="L47" s="17"/>
-      <c r="M47" s="17"/>
-      <c r="N47" s="17"/>
-      <c r="O47" s="17"/>
+      <c r="L47" s="6"/>
+      <c r="M47" s="22"/>
+      <c r="N47" s="22"/>
+      <c r="O47" s="22"/>
     </row>
     <row r="48" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B48" s="12"/>
       <c r="K48" s="13"/>
-      <c r="L48" s="17"/>
-      <c r="M48" s="17"/>
-      <c r="N48" s="17"/>
-      <c r="O48" s="17"/>
+      <c r="L48" s="6"/>
+      <c r="M48" s="22"/>
+      <c r="N48" s="22"/>
+      <c r="O48" s="22"/>
     </row>
     <row r="49" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B49" s="12"/>
       <c r="K49" s="13"/>
-      <c r="L49" s="17"/>
-      <c r="M49" s="17"/>
-      <c r="N49" s="17"/>
-      <c r="O49" s="17"/>
+      <c r="L49" s="6"/>
+      <c r="M49" s="22"/>
+      <c r="N49" s="22"/>
+      <c r="O49" s="22"/>
     </row>
     <row r="50" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B50" s="12"/>
       <c r="K50" s="13"/>
-      <c r="L50" s="17"/>
-      <c r="M50" s="17"/>
-      <c r="N50" s="17"/>
-      <c r="O50" s="17"/>
+      <c r="L50" s="6"/>
+      <c r="M50" s="22"/>
+      <c r="N50" s="22"/>
+      <c r="O50" s="22"/>
     </row>
     <row r="51" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B51" s="12"/>
       <c r="K51" s="13"/>
-      <c r="L51" s="17"/>
-      <c r="M51" s="17"/>
-      <c r="N51" s="17"/>
-      <c r="O51" s="17"/>
+      <c r="L51" s="6"/>
+      <c r="M51" s="22"/>
+      <c r="N51" s="22"/>
+      <c r="O51" s="22"/>
     </row>
     <row r="52" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B52" s="12"/>
       <c r="K52" s="13"/>
-      <c r="L52" s="17"/>
-      <c r="M52" s="17"/>
-      <c r="N52" s="17"/>
-      <c r="O52" s="17"/>
+      <c r="L52" s="6"/>
+      <c r="M52" s="22"/>
+      <c r="N52" s="22"/>
+      <c r="O52" s="22"/>
     </row>
     <row r="53" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B53" s="12"/>
       <c r="K53" s="13"/>
-      <c r="L53" s="17"/>
-      <c r="M53" s="17"/>
-      <c r="N53" s="17"/>
-      <c r="O53" s="17"/>
+      <c r="L53" s="6"/>
+      <c r="M53" s="22"/>
+      <c r="N53" s="22"/>
+      <c r="O53" s="22"/>
     </row>
     <row r="54" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B54" s="12"/>
       <c r="K54" s="13"/>
-      <c r="L54" s="17"/>
-      <c r="M54" s="17"/>
-      <c r="N54" s="17"/>
-      <c r="O54" s="17"/>
+      <c r="L54" s="6"/>
+      <c r="M54" s="22"/>
+      <c r="N54" s="22"/>
+      <c r="O54" s="22"/>
     </row>
     <row r="55" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B55" s="12"/>
       <c r="K55" s="13"/>
-      <c r="L55" s="17"/>
-      <c r="M55" s="17"/>
-      <c r="N55" s="17"/>
-      <c r="O55" s="17"/>
+      <c r="L55" s="6"/>
+      <c r="M55" s="22"/>
+      <c r="N55" s="22"/>
+      <c r="O55" s="22"/>
     </row>
     <row r="56" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B56" s="12"/>
       <c r="K56" s="13"/>
-      <c r="L56" s="17"/>
-      <c r="M56" s="17"/>
-      <c r="N56" s="17"/>
-      <c r="O56" s="17"/>
+      <c r="L56" s="6"/>
+      <c r="M56" s="22"/>
+      <c r="N56" s="22"/>
+      <c r="O56" s="22"/>
     </row>
     <row r="57" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B57" s="12"/>
       <c r="K57" s="13"/>
-      <c r="L57" s="17"/>
-      <c r="M57" s="17"/>
-      <c r="N57" s="17"/>
-      <c r="O57" s="17"/>
+      <c r="L57" s="6"/>
+      <c r="M57" s="22"/>
+      <c r="N57" s="22"/>
+      <c r="O57" s="22"/>
     </row>
     <row r="58" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B58" s="12"/>
       <c r="K58" s="13"/>
-      <c r="L58" s="17"/>
-      <c r="M58" s="17"/>
-      <c r="N58" s="17"/>
-      <c r="O58" s="17"/>
+      <c r="L58" s="6"/>
+      <c r="M58" s="22"/>
+      <c r="N58" s="22"/>
+      <c r="O58" s="22"/>
     </row>
     <row r="59" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B59" s="12"/>
       <c r="K59" s="13"/>
-      <c r="L59" s="17"/>
-      <c r="M59" s="17"/>
-      <c r="N59" s="17"/>
-      <c r="O59" s="17"/>
+      <c r="L59" s="6"/>
+      <c r="M59" s="22"/>
+      <c r="N59" s="22"/>
+      <c r="O59" s="22"/>
     </row>
     <row r="60" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B60" s="12"/>
       <c r="K60" s="13"/>
-      <c r="L60" s="17"/>
-      <c r="M60" s="17"/>
-      <c r="N60" s="17"/>
-      <c r="O60" s="17"/>
+      <c r="L60" s="6"/>
+      <c r="M60" s="22"/>
+      <c r="N60" s="22"/>
+      <c r="O60" s="22"/>
     </row>
     <row r="61" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B61" s="12"/>
       <c r="K61" s="13"/>
-      <c r="L61" s="17"/>
-      <c r="M61" s="17"/>
-      <c r="N61" s="17"/>
-      <c r="O61" s="17"/>
+      <c r="L61" s="6"/>
+      <c r="M61" s="22"/>
+      <c r="N61" s="22"/>
+      <c r="O61" s="22"/>
     </row>
     <row r="62" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B62" s="12"/>
       <c r="K62" s="13"/>
-      <c r="L62" s="17"/>
-      <c r="M62" s="17"/>
-      <c r="N62" s="17"/>
-      <c r="O62" s="17"/>
+      <c r="L62" s="6"/>
+      <c r="M62" s="22"/>
+      <c r="N62" s="22"/>
+      <c r="O62" s="22"/>
     </row>
     <row r="63" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B63" s="12"/>
       <c r="K63" s="13"/>
-      <c r="L63" s="17"/>
-      <c r="M63" s="17"/>
-      <c r="N63" s="17"/>
-      <c r="O63" s="17"/>
+      <c r="L63" s="6"/>
+      <c r="M63" s="22"/>
+      <c r="N63" s="22"/>
+      <c r="O63" s="22"/>
     </row>
     <row r="64" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B64" s="12"/>
       <c r="K64" s="13"/>
-      <c r="L64" s="17"/>
-      <c r="M64" s="17"/>
-      <c r="N64" s="17"/>
-      <c r="O64" s="17"/>
+      <c r="L64" s="6"/>
+      <c r="M64" s="22"/>
+      <c r="N64" s="22"/>
+      <c r="O64" s="22"/>
     </row>
     <row r="65" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B65" s="12"/>
       <c r="K65" s="13"/>
-      <c r="L65" s="17"/>
-      <c r="M65" s="17"/>
-      <c r="N65" s="17"/>
-      <c r="O65" s="17"/>
+      <c r="L65" s="6"/>
+      <c r="M65" s="22"/>
+      <c r="N65" s="22"/>
+      <c r="O65" s="22"/>
     </row>
     <row r="66" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B66" s="12"/>
       <c r="K66" s="13"/>
-      <c r="L66" s="17"/>
-      <c r="M66" s="17"/>
-      <c r="N66" s="17"/>
-      <c r="O66" s="17"/>
+      <c r="L66" s="6"/>
+      <c r="M66" s="22"/>
+      <c r="N66" s="22"/>
+      <c r="O66" s="22"/>
     </row>
     <row r="67" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B67" s="12"/>
       <c r="K67" s="13"/>
-      <c r="L67" s="17"/>
-      <c r="M67" s="17"/>
-      <c r="N67" s="17"/>
-      <c r="O67" s="17"/>
+      <c r="L67" s="6"/>
+      <c r="M67" s="22"/>
+      <c r="N67" s="22"/>
+      <c r="O67" s="22"/>
     </row>
     <row r="68" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B68" s="12"/>
       <c r="K68" s="13"/>
-      <c r="L68" s="17"/>
-      <c r="M68" s="17"/>
-      <c r="N68" s="17"/>
-      <c r="O68" s="17"/>
+      <c r="L68" s="6"/>
+      <c r="M68" s="22"/>
+      <c r="N68" s="22"/>
+      <c r="O68" s="22"/>
     </row>
     <row r="69" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B69" s="12"/>
       <c r="K69" s="13"/>
-      <c r="L69" s="17"/>
-      <c r="M69" s="17"/>
-      <c r="N69" s="17"/>
-      <c r="O69" s="17"/>
+      <c r="L69" s="6"/>
+      <c r="M69" s="22"/>
+      <c r="N69" s="22"/>
+      <c r="O69" s="22"/>
     </row>
     <row r="70" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B70" s="12"/>
       <c r="K70" s="13"/>
-      <c r="L70" s="17"/>
-      <c r="M70" s="17"/>
-      <c r="N70" s="17"/>
-      <c r="O70" s="17"/>
+      <c r="L70" s="6"/>
+      <c r="M70" s="22"/>
+      <c r="N70" s="22"/>
+      <c r="O70" s="22"/>
     </row>
     <row r="71" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B71" s="12"/>
       <c r="K71" s="13"/>
-      <c r="L71" s="17"/>
-      <c r="M71" s="17"/>
-      <c r="N71" s="17"/>
-      <c r="O71" s="17"/>
+      <c r="L71" s="6"/>
+      <c r="M71" s="22"/>
+      <c r="N71" s="22"/>
+      <c r="O71" s="22"/>
     </row>
     <row r="72" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B72" s="12"/>
       <c r="K72" s="13"/>
-      <c r="L72" s="17"/>
-      <c r="M72" s="17"/>
-      <c r="N72" s="17"/>
-      <c r="O72" s="17"/>
+      <c r="L72" s="6"/>
+      <c r="M72" s="22"/>
+      <c r="N72" s="22"/>
+      <c r="O72" s="22"/>
     </row>
     <row r="73" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B73" s="12"/>
       <c r="K73" s="13"/>
-      <c r="L73" s="17"/>
-      <c r="M73" s="17"/>
-      <c r="N73" s="17"/>
-      <c r="O73" s="17"/>
+      <c r="L73" s="6"/>
+      <c r="M73" s="22"/>
+      <c r="N73" s="22"/>
+      <c r="O73" s="22"/>
     </row>
     <row r="74" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B74" s="12"/>
       <c r="K74" s="13"/>
-      <c r="L74" s="17"/>
-      <c r="M74" s="17"/>
-      <c r="N74" s="17"/>
-      <c r="O74" s="17"/>
+      <c r="L74" s="6"/>
+      <c r="M74" s="22"/>
+      <c r="N74" s="22"/>
+      <c r="O74" s="22"/>
     </row>
     <row r="75" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B75" s="12"/>
       <c r="K75" s="13"/>
-      <c r="L75" s="17"/>
-      <c r="M75" s="17"/>
-      <c r="N75" s="17"/>
-      <c r="O75" s="17"/>
+      <c r="L75" s="6"/>
+      <c r="M75" s="22"/>
+      <c r="N75" s="22"/>
+      <c r="O75" s="22"/>
     </row>
     <row r="76" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B76" s="12"/>
       <c r="K76" s="13"/>
-      <c r="L76" s="17"/>
-      <c r="M76" s="17"/>
-      <c r="N76" s="17"/>
-      <c r="O76" s="17"/>
+      <c r="L76" s="6"/>
+      <c r="M76" s="22"/>
+      <c r="N76" s="22"/>
+      <c r="O76" s="22"/>
     </row>
     <row r="77" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B77" s="12"/>
       <c r="K77" s="13"/>
-      <c r="L77" s="21"/>
-      <c r="M77" s="20"/>
+      <c r="L77" s="17"/>
+      <c r="M77" s="23"/>
+      <c r="N77" s="23"/>
+      <c r="O77" s="23"/>
     </row>
     <row r="78" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B78" s="12"/>
-      <c r="C78" s="26"/>
-      <c r="D78" s="26"/>
-      <c r="E78" s="26"/>
-      <c r="F78" s="26"/>
-      <c r="G78" s="26"/>
-      <c r="H78" s="27"/>
-      <c r="I78" s="27"/>
-      <c r="J78" s="27"/>
+      <c r="H78" s="8"/>
+      <c r="I78" s="8"/>
+      <c r="J78" s="8"/>
       <c r="K78" s="13"/>
+      <c r="M78" s="23"/>
     </row>
     <row r="79" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B79" s="12"/>
-      <c r="C79" s="26"/>
-      <c r="D79" s="26"/>
-      <c r="E79" s="26"/>
-      <c r="F79" s="26"/>
-      <c r="G79" s="26"/>
-      <c r="H79" s="26"/>
-      <c r="I79" s="26"/>
-      <c r="J79" s="26"/>
       <c r="K79" s="13"/>
+      <c r="M79" s="23"/>
     </row>
     <row r="80" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B80" s="12"/>
@@ -7239,26 +7173,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="B1" t="s">
+      <c r="F1" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="24" t="s">
-        <v>23</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E1" s="24" t="s">
-        <v>25</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="G1" s="20" t="s">
         <v>27</v>
-      </c>
-      <c r="G1" s="24" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
bug 16: pdf chart
</commit_message>
<xml_diff>
--- a/web-console/server/assets/pdf_template.xlsx
+++ b/web-console/server/assets/pdf_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\DEV\UBA6\web-console\server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52BDB272-97B4-47CF-A21C-0C4D96146F4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A869A33E-9D32-4A31-9FF6-D76A159C517A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
   </bookViews>
   <sheets>
     <sheet name="Report" sheetId="1" r:id="rId1"/>
@@ -282,7 +282,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
@@ -319,8 +319,6 @@
     <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -399,13 +397,13 @@
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
         <c:ser>
-          <c:idx val="3"/>
-          <c:order val="0"/>
+          <c:idx val="0"/>
+          <c:order val="3"/>
           <c:tx>
             <c:v>Voltage [V]</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="9525" cap="rnd">
+            <a:ln w="25400" cap="rnd">
               <a:noFill/>
               <a:round/>
             </a:ln>
@@ -422,32 +420,26 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Data!$A$2:$A$50000</c:f>
+              <c:f>Data!$K$2:$K$500</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
+                <c:ptCount val="499"/>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Data!$C$2:$C$50000</c:f>
+              <c:f>Data!$L$2:$L$500</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
+                <c:ptCount val="499"/>
               </c:numCache>
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst>
+          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-71AD-41FA-AA0E-8879577C3941}"/>
+              <c16:uniqueId val="{00000003-71AD-41FA-AA0E-8879577C3941}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -463,6 +455,73 @@
         <c:axId val="538753616"/>
         <c:extLst>
           <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="3"/>
+                <c:order val="0"/>
+                <c:tx>
+                  <c:v>Voltage [V]</c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="9525" cap="rnd">
+                    <a:noFill/>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst>
+                    <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                      <a:srgbClr val="000000">
+                        <a:alpha val="63000"/>
+                      </a:srgbClr>
+                    </a:outerShdw>
+                  </a:effectLst>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>Data!$A$2:$A$50000</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="49999"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>Data!$C$2:$C$50000</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="49999"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000000-71AD-41FA-AA0E-8879577C3941}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
             <c15:filteredScatterSeries>
               <c15:ser>
                 <c:idx val="4"/>
@@ -490,8 +549,8 @@
                 </c:marker>
                 <c:xVal>
                   <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>[0]!Time</c15:sqref>
                         </c15:formulaRef>
@@ -508,8 +567,8 @@
                 </c:xVal>
                 <c:yVal>
                   <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>[0]!Temp</c15:sqref>
                         </c15:formulaRef>
@@ -525,7 +584,7 @@
                   </c:numRef>
                 </c:yVal>
                 <c:smooth val="0"/>
-                <c:extLst>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000001-71AD-41FA-AA0E-8879577C3941}"/>
                   </c:ext>
@@ -597,75 +656,6 @@
                 <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000002-71AD-41FA-AA0E-8879577C3941}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="0"/>
-                <c:order val="3"/>
-                <c:tx>
-                  <c:v>Voltage [V]</c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="9525" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent1"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst>
-                    <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                      <a:srgbClr val="000000">
-                        <a:alpha val="63000"/>
-                      </a:srgbClr>
-                    </a:outerShdw>
-                  </a:effectLst>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>Data!$A$2:$A$500</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="499"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>Data!$C$2:$C$500</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="499"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000003-71AD-41FA-AA0E-8879577C3941}"/>
                   </c:ext>
                 </c:extLst>
               </c15:ser>
@@ -933,19 +923,16 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Data!$A$2:$A$50000</c:f>
+              <c:f>Data!$K$2:$K$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Data!$H$2:$H$50000</c:f>
+              <c:f>Data!$L$2:$L$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="49999"/>
@@ -1487,25 +1474,19 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Data!$A$2:$A$50000</c:f>
+              <c:f>Data!$K$2:$K$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Data!$E$2:$E$50000</c:f>
+              <c:f>Data!$N$2:$N$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -1850,7 +1831,10 @@
           <c:spPr>
             <a:ln w="12700" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="tx1"/>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="50000"/>
+                  <a:lumOff val="50000"/>
+                </a:schemeClr>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -1861,25 +1845,19 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Data!$A$2:$A$50000</c:f>
+              <c:f>Data!$K$2:$K$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Data!$C$2:$C$50000</c:f>
+              <c:f>Data!$L$2:$L$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -1973,9 +1951,12 @@
                   <c:v>Voltage [V]</c:v>
                 </c:tx>
                 <c:spPr>
-                  <a:ln w="15875" cap="rnd">
+                  <a:ln w="12700" cap="rnd">
                     <a:solidFill>
-                      <a:schemeClr val="accent1"/>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="50000"/>
+                        <a:lumOff val="50000"/>
+                      </a:schemeClr>
                     </a:solidFill>
                     <a:round/>
                   </a:ln>
@@ -2117,25 +2098,19 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Data!$A$2:$A$50000</c:f>
+              <c:f>Data!$K$2:$K$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Data!$D$2:$D$50000</c:f>
+              <c:f>Data!$M$2:$M$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -2503,10 +2478,8 @@
             <c:v>Temprture [°C]</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="12700" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -2516,25 +2489,19 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Data!$A$2:$A$50000</c:f>
+              <c:f>Data!$K$2:$K$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Data!$E$2:$E$50000</c:f>
+              <c:f>Data!$N$2:$N$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -5763,8 +5730,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="609732" y="402938"/>
-          <a:ext cx="9277828" cy="4213844"/>
+          <a:off x="605922" y="396588"/>
+          <a:ext cx="9312753" cy="4137009"/>
           <a:chOff x="614350" y="401783"/>
           <a:chExt cx="9325165" cy="4265799"/>
         </a:xfrm>
@@ -6572,9 +6539,6 @@
       <c r="J28" s="8"/>
       <c r="K28" s="9"/>
       <c r="L28" s="17"/>
-      <c r="M28" s="23"/>
-      <c r="N28" s="23"/>
-      <c r="O28" s="23"/>
     </row>
     <row r="29" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B29" s="12"/>
@@ -6587,9 +6551,6 @@
       <c r="I29" s="19"/>
       <c r="K29" s="13"/>
       <c r="L29" s="17"/>
-      <c r="M29" s="23"/>
-      <c r="N29" s="23"/>
-      <c r="O29" s="23"/>
     </row>
     <row r="30" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B30" s="12"/>
@@ -6599,9 +6560,9 @@
       <c r="I30" s="19"/>
       <c r="K30" s="13"/>
       <c r="L30" s="6"/>
-      <c r="M30" s="22"/>
-      <c r="N30" s="22"/>
-      <c r="O30" s="22"/>
+      <c r="M30" s="8"/>
+      <c r="N30" s="8"/>
+      <c r="O30" s="8"/>
     </row>
     <row r="31" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B31" s="12"/>
@@ -6614,9 +6575,9 @@
       <c r="I31" s="19"/>
       <c r="K31" s="13"/>
       <c r="L31" s="6"/>
-      <c r="M31" s="22"/>
-      <c r="N31" s="22"/>
-      <c r="O31" s="22"/>
+      <c r="M31" s="8"/>
+      <c r="N31" s="8"/>
+      <c r="O31" s="8"/>
     </row>
     <row r="32" spans="2:15" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B32" s="6"/>
@@ -6635,9 +6596,6 @@
       </c>
       <c r="K32" s="9"/>
       <c r="L32" s="6"/>
-      <c r="M32" s="22"/>
-      <c r="N32" s="22"/>
-      <c r="O32" s="22"/>
     </row>
     <row r="33" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B33" s="12"/>
@@ -6650,9 +6608,9 @@
       </c>
       <c r="K33" s="13"/>
       <c r="L33" s="6"/>
-      <c r="M33" s="22"/>
-      <c r="N33" s="22"/>
-      <c r="O33" s="22"/>
+      <c r="M33" s="8"/>
+      <c r="N33" s="8"/>
+      <c r="O33" s="8"/>
     </row>
     <row r="34" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B34" s="12"/>
@@ -6665,9 +6623,9 @@
       </c>
       <c r="K34" s="13"/>
       <c r="L34" s="6"/>
-      <c r="M34" s="22"/>
-      <c r="N34" s="22"/>
-      <c r="O34" s="22"/>
+      <c r="M34" s="8"/>
+      <c r="N34" s="8"/>
+      <c r="O34" s="8"/>
     </row>
     <row r="35" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B35" s="12"/>
@@ -6677,9 +6635,9 @@
       <c r="I35" s="19"/>
       <c r="K35" s="13"/>
       <c r="L35" s="6"/>
-      <c r="M35" s="22"/>
-      <c r="N35" s="22"/>
-      <c r="O35" s="22"/>
+      <c r="M35" s="8"/>
+      <c r="N35" s="8"/>
+      <c r="O35" s="8"/>
     </row>
     <row r="36" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B36" s="12"/>
@@ -6692,9 +6650,9 @@
       <c r="I36" s="19"/>
       <c r="K36" s="13"/>
       <c r="L36" s="6"/>
-      <c r="M36" s="22"/>
-      <c r="N36" s="22"/>
-      <c r="O36" s="22"/>
+      <c r="M36" s="8"/>
+      <c r="N36" s="8"/>
+      <c r="O36" s="8"/>
     </row>
     <row r="37" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B37" s="12"/>
@@ -6707,9 +6665,9 @@
       <c r="I37" s="19"/>
       <c r="K37" s="13"/>
       <c r="L37" s="6"/>
-      <c r="M37" s="22"/>
-      <c r="N37" s="22"/>
-      <c r="O37" s="22"/>
+      <c r="M37" s="8"/>
+      <c r="N37" s="8"/>
+      <c r="O37" s="8"/>
     </row>
     <row r="38" spans="2:15" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B38" s="6"/>
@@ -6718,9 +6676,6 @@
       </c>
       <c r="K38" s="9"/>
       <c r="L38" s="6"/>
-      <c r="M38" s="22"/>
-      <c r="N38" s="22"/>
-      <c r="O38" s="22"/>
     </row>
     <row r="39" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B39" s="12"/>
@@ -6733,17 +6688,17 @@
       <c r="J39" s="21"/>
       <c r="K39" s="13"/>
       <c r="L39" s="6"/>
-      <c r="M39" s="22"/>
-      <c r="N39" s="22"/>
-      <c r="O39" s="22"/>
+      <c r="M39" s="8"/>
+      <c r="N39" s="8"/>
+      <c r="O39" s="8"/>
     </row>
     <row r="40" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B40" s="12"/>
       <c r="K40" s="13"/>
       <c r="L40" s="6"/>
-      <c r="M40" s="22"/>
-      <c r="N40" s="22"/>
-      <c r="O40" s="22"/>
+      <c r="M40" s="8"/>
+      <c r="N40" s="8"/>
+      <c r="O40" s="8"/>
     </row>
     <row r="41" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B41" s="12"/>
@@ -6759,297 +6714,294 @@
       <c r="J41" s="8"/>
       <c r="K41" s="13"/>
       <c r="L41" s="6"/>
-      <c r="M41" s="22"/>
-      <c r="N41" s="22"/>
-      <c r="O41" s="22"/>
+      <c r="M41" s="8"/>
+      <c r="N41" s="8"/>
+      <c r="O41" s="8"/>
     </row>
     <row r="42" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B42" s="12"/>
       <c r="K42" s="13"/>
       <c r="L42" s="6"/>
-      <c r="M42" s="22"/>
-      <c r="N42" s="22"/>
-      <c r="O42" s="22"/>
+      <c r="M42" s="8"/>
+      <c r="N42" s="8"/>
+      <c r="O42" s="8"/>
     </row>
     <row r="43" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B43" s="12"/>
       <c r="K43" s="13"/>
       <c r="L43" s="6"/>
-      <c r="M43" s="22"/>
-      <c r="N43" s="22"/>
-      <c r="O43" s="22"/>
+      <c r="M43" s="8"/>
+      <c r="N43" s="8"/>
+      <c r="O43" s="8"/>
     </row>
     <row r="44" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B44" s="12"/>
       <c r="K44" s="13"/>
       <c r="L44" s="6"/>
-      <c r="M44" s="22"/>
-      <c r="N44" s="22"/>
-      <c r="O44" s="22"/>
+      <c r="M44" s="8"/>
+      <c r="N44" s="8"/>
+      <c r="O44" s="8"/>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B45" s="12"/>
       <c r="K45" s="13"/>
       <c r="L45" s="6"/>
-      <c r="M45" s="22"/>
-      <c r="N45" s="22"/>
-      <c r="O45" s="22"/>
+      <c r="M45" s="8"/>
+      <c r="N45" s="8"/>
+      <c r="O45" s="8"/>
     </row>
     <row r="46" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="12"/>
       <c r="K46" s="13"/>
       <c r="L46" s="6"/>
-      <c r="M46" s="22"/>
-      <c r="N46" s="22"/>
-      <c r="O46" s="22"/>
+      <c r="M46" s="8"/>
+      <c r="N46" s="8"/>
+      <c r="O46" s="8"/>
     </row>
     <row r="47" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="12"/>
       <c r="K47" s="13"/>
       <c r="L47" s="6"/>
-      <c r="M47" s="22"/>
-      <c r="N47" s="22"/>
-      <c r="O47" s="22"/>
+      <c r="M47" s="8"/>
+      <c r="N47" s="8"/>
+      <c r="O47" s="8"/>
     </row>
     <row r="48" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B48" s="12"/>
       <c r="K48" s="13"/>
       <c r="L48" s="6"/>
-      <c r="M48" s="22"/>
-      <c r="N48" s="22"/>
-      <c r="O48" s="22"/>
+      <c r="M48" s="8"/>
+      <c r="N48" s="8"/>
+      <c r="O48" s="8"/>
     </row>
     <row r="49" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B49" s="12"/>
       <c r="K49" s="13"/>
       <c r="L49" s="6"/>
-      <c r="M49" s="22"/>
-      <c r="N49" s="22"/>
-      <c r="O49" s="22"/>
+      <c r="M49" s="8"/>
+      <c r="N49" s="8"/>
+      <c r="O49" s="8"/>
     </row>
     <row r="50" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B50" s="12"/>
       <c r="K50" s="13"/>
       <c r="L50" s="6"/>
-      <c r="M50" s="22"/>
-      <c r="N50" s="22"/>
-      <c r="O50" s="22"/>
+      <c r="M50" s="8"/>
+      <c r="N50" s="8"/>
+      <c r="O50" s="8"/>
     </row>
     <row r="51" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B51" s="12"/>
       <c r="K51" s="13"/>
       <c r="L51" s="6"/>
-      <c r="M51" s="22"/>
-      <c r="N51" s="22"/>
-      <c r="O51" s="22"/>
+      <c r="M51" s="8"/>
+      <c r="N51" s="8"/>
+      <c r="O51" s="8"/>
     </row>
     <row r="52" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B52" s="12"/>
       <c r="K52" s="13"/>
       <c r="L52" s="6"/>
-      <c r="M52" s="22"/>
-      <c r="N52" s="22"/>
-      <c r="O52" s="22"/>
+      <c r="M52" s="8"/>
+      <c r="N52" s="8"/>
+      <c r="O52" s="8"/>
     </row>
     <row r="53" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B53" s="12"/>
       <c r="K53" s="13"/>
       <c r="L53" s="6"/>
-      <c r="M53" s="22"/>
-      <c r="N53" s="22"/>
-      <c r="O53" s="22"/>
+      <c r="M53" s="8"/>
+      <c r="N53" s="8"/>
+      <c r="O53" s="8"/>
     </row>
     <row r="54" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B54" s="12"/>
       <c r="K54" s="13"/>
       <c r="L54" s="6"/>
-      <c r="M54" s="22"/>
-      <c r="N54" s="22"/>
-      <c r="O54" s="22"/>
+      <c r="M54" s="8"/>
+      <c r="N54" s="8"/>
+      <c r="O54" s="8"/>
     </row>
     <row r="55" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B55" s="12"/>
       <c r="K55" s="13"/>
       <c r="L55" s="6"/>
-      <c r="M55" s="22"/>
-      <c r="N55" s="22"/>
-      <c r="O55" s="22"/>
+      <c r="M55" s="8"/>
+      <c r="N55" s="8"/>
+      <c r="O55" s="8"/>
     </row>
     <row r="56" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B56" s="12"/>
       <c r="K56" s="13"/>
       <c r="L56" s="6"/>
-      <c r="M56" s="22"/>
-      <c r="N56" s="22"/>
-      <c r="O56" s="22"/>
+      <c r="M56" s="8"/>
+      <c r="N56" s="8"/>
+      <c r="O56" s="8"/>
     </row>
     <row r="57" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B57" s="12"/>
       <c r="K57" s="13"/>
       <c r="L57" s="6"/>
-      <c r="M57" s="22"/>
-      <c r="N57" s="22"/>
-      <c r="O57" s="22"/>
+      <c r="M57" s="8"/>
+      <c r="N57" s="8"/>
+      <c r="O57" s="8"/>
     </row>
     <row r="58" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B58" s="12"/>
       <c r="K58" s="13"/>
       <c r="L58" s="6"/>
-      <c r="M58" s="22"/>
-      <c r="N58" s="22"/>
-      <c r="O58" s="22"/>
+      <c r="M58" s="8"/>
+      <c r="N58" s="8"/>
+      <c r="O58" s="8"/>
     </row>
     <row r="59" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B59" s="12"/>
       <c r="K59" s="13"/>
       <c r="L59" s="6"/>
-      <c r="M59" s="22"/>
-      <c r="N59" s="22"/>
-      <c r="O59" s="22"/>
+      <c r="M59" s="8"/>
+      <c r="N59" s="8"/>
+      <c r="O59" s="8"/>
     </row>
     <row r="60" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B60" s="12"/>
       <c r="K60" s="13"/>
       <c r="L60" s="6"/>
-      <c r="M60" s="22"/>
-      <c r="N60" s="22"/>
-      <c r="O60" s="22"/>
+      <c r="M60" s="8"/>
+      <c r="N60" s="8"/>
+      <c r="O60" s="8"/>
     </row>
     <row r="61" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B61" s="12"/>
       <c r="K61" s="13"/>
       <c r="L61" s="6"/>
-      <c r="M61" s="22"/>
-      <c r="N61" s="22"/>
-      <c r="O61" s="22"/>
+      <c r="M61" s="8"/>
+      <c r="N61" s="8"/>
+      <c r="O61" s="8"/>
     </row>
     <row r="62" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B62" s="12"/>
       <c r="K62" s="13"/>
       <c r="L62" s="6"/>
-      <c r="M62" s="22"/>
-      <c r="N62" s="22"/>
-      <c r="O62" s="22"/>
+      <c r="M62" s="8"/>
+      <c r="N62" s="8"/>
+      <c r="O62" s="8"/>
     </row>
     <row r="63" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B63" s="12"/>
       <c r="K63" s="13"/>
       <c r="L63" s="6"/>
-      <c r="M63" s="22"/>
-      <c r="N63" s="22"/>
-      <c r="O63" s="22"/>
+      <c r="M63" s="8"/>
+      <c r="N63" s="8"/>
+      <c r="O63" s="8"/>
     </row>
     <row r="64" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B64" s="12"/>
       <c r="K64" s="13"/>
       <c r="L64" s="6"/>
-      <c r="M64" s="22"/>
-      <c r="N64" s="22"/>
-      <c r="O64" s="22"/>
+      <c r="M64" s="8"/>
+      <c r="N64" s="8"/>
+      <c r="O64" s="8"/>
     </row>
     <row r="65" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B65" s="12"/>
       <c r="K65" s="13"/>
       <c r="L65" s="6"/>
-      <c r="M65" s="22"/>
-      <c r="N65" s="22"/>
-      <c r="O65" s="22"/>
+      <c r="M65" s="8"/>
+      <c r="N65" s="8"/>
+      <c r="O65" s="8"/>
     </row>
     <row r="66" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B66" s="12"/>
       <c r="K66" s="13"/>
       <c r="L66" s="6"/>
-      <c r="M66" s="22"/>
-      <c r="N66" s="22"/>
-      <c r="O66" s="22"/>
+      <c r="M66" s="8"/>
+      <c r="N66" s="8"/>
+      <c r="O66" s="8"/>
     </row>
     <row r="67" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B67" s="12"/>
       <c r="K67" s="13"/>
       <c r="L67" s="6"/>
-      <c r="M67" s="22"/>
-      <c r="N67" s="22"/>
-      <c r="O67" s="22"/>
+      <c r="M67" s="8"/>
+      <c r="N67" s="8"/>
+      <c r="O67" s="8"/>
     </row>
     <row r="68" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B68" s="12"/>
       <c r="K68" s="13"/>
       <c r="L68" s="6"/>
-      <c r="M68" s="22"/>
-      <c r="N68" s="22"/>
-      <c r="O68" s="22"/>
+      <c r="M68" s="8"/>
+      <c r="N68" s="8"/>
+      <c r="O68" s="8"/>
     </row>
     <row r="69" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B69" s="12"/>
       <c r="K69" s="13"/>
       <c r="L69" s="6"/>
-      <c r="M69" s="22"/>
-      <c r="N69" s="22"/>
-      <c r="O69" s="22"/>
+      <c r="M69" s="8"/>
+      <c r="N69" s="8"/>
+      <c r="O69" s="8"/>
     </row>
     <row r="70" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B70" s="12"/>
       <c r="K70" s="13"/>
       <c r="L70" s="6"/>
-      <c r="M70" s="22"/>
-      <c r="N70" s="22"/>
-      <c r="O70" s="22"/>
+      <c r="M70" s="8"/>
+      <c r="N70" s="8"/>
+      <c r="O70" s="8"/>
     </row>
     <row r="71" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B71" s="12"/>
       <c r="K71" s="13"/>
       <c r="L71" s="6"/>
-      <c r="M71" s="22"/>
-      <c r="N71" s="22"/>
-      <c r="O71" s="22"/>
+      <c r="M71" s="8"/>
+      <c r="N71" s="8"/>
+      <c r="O71" s="8"/>
     </row>
     <row r="72" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B72" s="12"/>
       <c r="K72" s="13"/>
       <c r="L72" s="6"/>
-      <c r="M72" s="22"/>
-      <c r="N72" s="22"/>
-      <c r="O72" s="22"/>
+      <c r="M72" s="8"/>
+      <c r="N72" s="8"/>
+      <c r="O72" s="8"/>
     </row>
     <row r="73" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B73" s="12"/>
       <c r="K73" s="13"/>
       <c r="L73" s="6"/>
-      <c r="M73" s="22"/>
-      <c r="N73" s="22"/>
-      <c r="O73" s="22"/>
+      <c r="M73" s="8"/>
+      <c r="N73" s="8"/>
+      <c r="O73" s="8"/>
     </row>
     <row r="74" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B74" s="12"/>
       <c r="K74" s="13"/>
       <c r="L74" s="6"/>
-      <c r="M74" s="22"/>
-      <c r="N74" s="22"/>
-      <c r="O74" s="22"/>
+      <c r="M74" s="8"/>
+      <c r="N74" s="8"/>
+      <c r="O74" s="8"/>
     </row>
     <row r="75" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B75" s="12"/>
       <c r="K75" s="13"/>
       <c r="L75" s="6"/>
-      <c r="M75" s="22"/>
-      <c r="N75" s="22"/>
-      <c r="O75" s="22"/>
+      <c r="M75" s="8"/>
+      <c r="N75" s="8"/>
+      <c r="O75" s="8"/>
     </row>
     <row r="76" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B76" s="12"/>
       <c r="K76" s="13"/>
       <c r="L76" s="6"/>
-      <c r="M76" s="22"/>
-      <c r="N76" s="22"/>
-      <c r="O76" s="22"/>
+      <c r="M76" s="8"/>
+      <c r="N76" s="8"/>
+      <c r="O76" s="8"/>
     </row>
     <row r="77" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B77" s="12"/>
       <c r="K77" s="13"/>
       <c r="L77" s="17"/>
-      <c r="M77" s="23"/>
-      <c r="N77" s="23"/>
-      <c r="O77" s="23"/>
     </row>
     <row r="78" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B78" s="12"/>
@@ -7057,12 +7009,10 @@
       <c r="I78" s="8"/>
       <c r="J78" s="8"/>
       <c r="K78" s="13"/>
-      <c r="M78" s="23"/>
     </row>
     <row r="79" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B79" s="12"/>
       <c r="K79" s="13"/>
-      <c r="M79" s="23"/>
     </row>
     <row r="80" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B80" s="12"/>

</xml_diff>

<commit_message>
pdf template - separate pages, correction in service Worker
</commit_message>
<xml_diff>
--- a/web-console/server/assets/pdf_template.xlsx
+++ b/web-console/server/assets/pdf_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\DEV\UBA6\web-console\server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A869A33E-9D32-4A31-9FF6-D76A159C517A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9405F6C-6F14-491E-8CB2-E88E31A50346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
   </bookViews>
@@ -196,83 +196,19 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="7">
+  <borders count="1">
     <border>
       <left/>
       <right/>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -282,33 +218,22 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
@@ -316,8 +241,13 @@
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -5730,7 +5660,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="605922" y="396588"/>
+          <a:off x="605922" y="380713"/>
           <a:ext cx="9312753" cy="4137009"/>
           <a:chOff x="614350" y="401783"/>
           <a:chExt cx="9325165" cy="4265799"/>
@@ -6193,7 +6123,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:O100"/>
+  <dimension ref="B1:O143"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.44140625" style="2" customWidth="1"/>
@@ -6202,908 +6132,1125 @@
     <col min="4" max="9" width="19.6640625" style="2" customWidth="1"/>
     <col min="10" max="10" width="9.44140625" style="2" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="4.109375" style="2" customWidth="1"/>
-    <col min="12" max="12" width="9.109375" style="15"/>
+    <col min="12" max="12" width="9.109375" style="8"/>
     <col min="13" max="13" width="82.44140625" style="2" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="123.33203125" style="2" customWidth="1"/>
     <col min="15" max="15" width="78.88671875" style="2" customWidth="1"/>
     <col min="16" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="J1" s="16"/>
+    <row r="1" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
     </row>
     <row r="2" spans="2:14" ht="8.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="3"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="5"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="14"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B3" s="6"/>
-      <c r="D3" s="7" t="s">
+      <c r="B3" s="13"/>
+      <c r="D3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="8"/>
-      <c r="F3" s="7" t="s">
+      <c r="E3" s="4"/>
+      <c r="F3" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="J3" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="K3" s="9"/>
-      <c r="N3" s="10"/>
+      <c r="K3" s="13"/>
+      <c r="N3" s="5"/>
     </row>
     <row r="4" spans="2:14" ht="5.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="6"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="8"/>
-      <c r="K4" s="9"/>
-      <c r="N4" s="10"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="13"/>
+      <c r="K4" s="13"/>
+      <c r="N4" s="5"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B5" s="12"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="18"/>
-      <c r="J5" s="18"/>
-      <c r="K5" s="13"/>
+      <c r="B5" s="14"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="14"/>
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B6" s="12"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="18"/>
-      <c r="J6" s="18"/>
-      <c r="K6" s="13"/>
+      <c r="B6" s="14"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="15"/>
+      <c r="K6" s="14"/>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B7" s="12"/>
-      <c r="C7" s="18"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18"/>
-      <c r="I7" s="18"/>
-      <c r="J7" s="18"/>
-      <c r="K7" s="13"/>
+      <c r="B7" s="14"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="15"/>
+      <c r="K7" s="14"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B8" s="12"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18"/>
-      <c r="H8" s="18"/>
-      <c r="I8" s="18"/>
-      <c r="J8" s="18"/>
-      <c r="K8" s="13"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="9"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="14"/>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B9" s="12"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="18"/>
-      <c r="H9" s="18"/>
-      <c r="I9" s="18"/>
-      <c r="J9" s="18"/>
-      <c r="K9" s="13"/>
+      <c r="B9" s="14"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="9"/>
+      <c r="J9" s="15"/>
+      <c r="K9" s="14"/>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B10" s="12"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
-      <c r="G10" s="18"/>
-      <c r="H10" s="18"/>
-      <c r="I10" s="18"/>
-      <c r="J10" s="18"/>
-      <c r="K10" s="13"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="9"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="14"/>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B11" s="12"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
-      <c r="G11" s="18"/>
-      <c r="H11" s="18"/>
-      <c r="I11" s="18"/>
-      <c r="J11" s="18"/>
-      <c r="K11" s="13"/>
+      <c r="B11" s="14"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="14"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B12" s="12"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="18"/>
-      <c r="I12" s="18"/>
-      <c r="J12" s="18"/>
-      <c r="K12" s="13"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="9"/>
+      <c r="J12" s="15"/>
+      <c r="K12" s="14"/>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B13" s="12"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="18"/>
-      <c r="J13" s="18"/>
-      <c r="K13" s="13"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="15"/>
+      <c r="K13" s="14"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B14" s="12"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
-      <c r="I14" s="18"/>
-      <c r="J14" s="18"/>
-      <c r="K14" s="13"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="15"/>
+      <c r="K14" s="14"/>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B15" s="12"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
-      <c r="G15" s="18"/>
-      <c r="H15" s="18"/>
-      <c r="I15" s="18"/>
-      <c r="J15" s="18"/>
-      <c r="K15" s="13"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="15"/>
+      <c r="K15" s="14"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B16" s="12"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="18"/>
-      <c r="H16" s="18"/>
-      <c r="I16" s="18"/>
-      <c r="J16" s="18"/>
-      <c r="K16" s="13"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
+      <c r="J16" s="15"/>
+      <c r="K16" s="14"/>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B17" s="12"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18"/>
-      <c r="H17" s="18"/>
-      <c r="I17" s="18"/>
-      <c r="J17" s="18"/>
-      <c r="K17" s="13"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="15"/>
+      <c r="K17" s="14"/>
     </row>
     <row r="18" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B18" s="12"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="18"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18"/>
-      <c r="I18" s="18"/>
-      <c r="J18" s="18"/>
-      <c r="K18" s="13"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="9"/>
+      <c r="J18" s="15"/>
+      <c r="K18" s="14"/>
     </row>
     <row r="19" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B19" s="12"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
-      <c r="I19" s="18"/>
-      <c r="J19" s="18"/>
-      <c r="K19" s="13"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="9"/>
+      <c r="J19" s="15"/>
+      <c r="K19" s="14"/>
     </row>
     <row r="20" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B20" s="12"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="18"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="18"/>
-      <c r="I20" s="18"/>
-      <c r="J20" s="18"/>
-      <c r="K20" s="13"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="9"/>
+      <c r="J20" s="15"/>
+      <c r="K20" s="14"/>
     </row>
     <row r="21" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B21" s="12"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="18"/>
-      <c r="G21" s="18"/>
-      <c r="H21" s="18"/>
-      <c r="I21" s="18"/>
-      <c r="J21" s="18"/>
-      <c r="K21" s="13"/>
+      <c r="B21" s="14"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="15"/>
+      <c r="K21" s="14"/>
     </row>
     <row r="22" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B22" s="12"/>
-      <c r="C22" s="18"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="18"/>
-      <c r="F22" s="18"/>
-      <c r="G22" s="18"/>
-      <c r="H22" s="18"/>
-      <c r="I22" s="18"/>
-      <c r="J22" s="18"/>
-      <c r="K22" s="13"/>
+      <c r="B22" s="14"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
+      <c r="J22" s="15"/>
+      <c r="K22" s="14"/>
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B23" s="12"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="18"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="18"/>
-      <c r="H23" s="18"/>
-      <c r="I23" s="18"/>
-      <c r="J23" s="18"/>
-      <c r="K23" s="13"/>
+      <c r="B23" s="14"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
+      <c r="I23" s="9"/>
+      <c r="J23" s="15"/>
+      <c r="K23" s="14"/>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B24" s="12"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="18"/>
-      <c r="F24" s="18"/>
-      <c r="G24" s="18"/>
-      <c r="H24" s="18"/>
-      <c r="I24" s="18"/>
-      <c r="J24" s="18"/>
-      <c r="K24" s="13"/>
+      <c r="B24" s="14"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
+      <c r="I24" s="9"/>
+      <c r="J24" s="15"/>
+      <c r="K24" s="14"/>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B25" s="12"/>
-      <c r="C25" s="18"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18"/>
-      <c r="F25" s="18"/>
-      <c r="G25" s="18"/>
-      <c r="H25" s="18"/>
-      <c r="I25" s="18"/>
-      <c r="J25" s="18"/>
-      <c r="K25" s="13"/>
+      <c r="B25" s="14"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
+      <c r="I25" s="9"/>
+      <c r="J25" s="15"/>
+      <c r="K25" s="14"/>
     </row>
     <row r="26" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B26" s="12"/>
-      <c r="C26" s="18"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="18"/>
-      <c r="G26" s="18"/>
-      <c r="H26" s="18"/>
-      <c r="I26" s="18"/>
-      <c r="J26" s="18"/>
-      <c r="K26" s="13"/>
-      <c r="M26" s="14"/>
+      <c r="B26" s="14"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
+      <c r="I26" s="9"/>
+      <c r="J26" s="15"/>
+      <c r="K26" s="14"/>
+      <c r="M26" s="7"/>
     </row>
     <row r="27" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B27" s="12"/>
-      <c r="K27" s="13"/>
+      <c r="B27" s="14"/>
+      <c r="J27" s="14"/>
+      <c r="K27" s="14"/>
     </row>
     <row r="28" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B28" s="6"/>
-      <c r="D28" s="8" t="s">
+      <c r="B28" s="13"/>
+      <c r="J28" s="14"/>
+      <c r="K28" s="13"/>
+      <c r="L28" s="12"/>
+    </row>
+    <row r="29" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B29" s="14"/>
+      <c r="D29" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E28" s="8"/>
-      <c r="F28" s="8"/>
-      <c r="G28" s="8"/>
-      <c r="H28" s="8" t="s">
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="I28" s="8"/>
-      <c r="J28" s="8"/>
-      <c r="K28" s="9"/>
-      <c r="L28" s="17"/>
-    </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B29" s="12"/>
-      <c r="D29" s="2" t="s">
+      <c r="I29" s="4"/>
+      <c r="J29" s="13"/>
+      <c r="K29" s="14"/>
+      <c r="L29" s="12"/>
+    </row>
+    <row r="30" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B30" s="14"/>
+      <c r="D30" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H29" s="2" t="s">
+      <c r="H30" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I29" s="19"/>
-      <c r="K29" s="13"/>
-      <c r="L29" s="17"/>
-    </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B30" s="12"/>
-      <c r="H30" s="2" t="s">
+      <c r="I30" s="10"/>
+      <c r="J30" s="14"/>
+      <c r="K30" s="14"/>
+      <c r="L30" s="13"/>
+      <c r="M30" s="4"/>
+      <c r="N30" s="4"/>
+      <c r="O30" s="4"/>
+    </row>
+    <row r="31" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B31" s="14"/>
+      <c r="H31" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I30" s="19"/>
-      <c r="K30" s="13"/>
-      <c r="L30" s="6"/>
-      <c r="M30" s="8"/>
-      <c r="N30" s="8"/>
-      <c r="O30" s="8"/>
-    </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B31" s="12"/>
-      <c r="D31" s="2" t="s">
+      <c r="I31" s="10"/>
+      <c r="J31" s="14"/>
+      <c r="K31" s="14"/>
+      <c r="L31" s="13"/>
+      <c r="M31" s="4"/>
+      <c r="N31" s="4"/>
+      <c r="O31" s="4"/>
+    </row>
+    <row r="32" spans="2:15" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="13"/>
+      <c r="D32" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="H31" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="I31" s="19"/>
-      <c r="K31" s="13"/>
-      <c r="L31" s="6"/>
-      <c r="M31" s="8"/>
-      <c r="N31" s="8"/>
-      <c r="O31" s="8"/>
-    </row>
-    <row r="32" spans="2:15" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="6"/>
-      <c r="D32" s="2" t="s">
-        <v>10</v>
       </c>
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
       <c r="H32" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I32" s="10"/>
+      <c r="J32" s="14"/>
+      <c r="K32" s="13"/>
+      <c r="L32" s="13"/>
+    </row>
+    <row r="33" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B33" s="14"/>
+      <c r="D33" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H33" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I32" s="19"/>
-      <c r="J32" s="2" t="s">
+      <c r="I33" s="10"/>
+      <c r="J33" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="K32" s="9"/>
-      <c r="L32" s="6"/>
-    </row>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B33" s="12"/>
-      <c r="H33" s="2" t="s">
+      <c r="K33" s="14"/>
+      <c r="L33" s="13"/>
+      <c r="M33" s="4"/>
+      <c r="N33" s="4"/>
+      <c r="O33" s="4"/>
+    </row>
+    <row r="34" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B34" s="14"/>
+      <c r="H34" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="I33" s="19"/>
-      <c r="J33" s="2" t="s">
+      <c r="I34" s="10"/>
+      <c r="J34" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="K33" s="13"/>
-      <c r="L33" s="6"/>
-      <c r="M33" s="8"/>
-      <c r="N33" s="8"/>
-      <c r="O33" s="8"/>
-    </row>
-    <row r="34" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B34" s="12"/>
-      <c r="H34" s="2" t="s">
+      <c r="K34" s="14"/>
+      <c r="L34" s="13"/>
+      <c r="M34" s="4"/>
+      <c r="N34" s="4"/>
+      <c r="O34" s="4"/>
+    </row>
+    <row r="35" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B35" s="14"/>
+      <c r="H35" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="I34" s="19"/>
-      <c r="J34" s="2" t="s">
+      <c r="I35" s="10"/>
+      <c r="J35" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="K34" s="13"/>
-      <c r="L34" s="6"/>
-      <c r="M34" s="8"/>
-      <c r="N34" s="8"/>
-      <c r="O34" s="8"/>
-    </row>
-    <row r="35" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B35" s="12"/>
-      <c r="H35" s="2" t="s">
+      <c r="K35" s="14"/>
+      <c r="L35" s="13"/>
+      <c r="M35" s="4"/>
+      <c r="N35" s="4"/>
+      <c r="O35" s="4"/>
+    </row>
+    <row r="36" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B36" s="14"/>
+      <c r="H36" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I35" s="19"/>
-      <c r="K35" s="13"/>
-      <c r="L35" s="6"/>
-      <c r="M35" s="8"/>
-      <c r="N35" s="8"/>
-      <c r="O35" s="8"/>
-    </row>
-    <row r="36" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B36" s="12"/>
-      <c r="D36" s="2" t="s">
+      <c r="I36" s="10"/>
+      <c r="J36" s="14"/>
+      <c r="K36" s="14"/>
+      <c r="L36" s="13"/>
+      <c r="M36" s="4"/>
+      <c r="N36" s="4"/>
+      <c r="O36" s="4"/>
+    </row>
+    <row r="37" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B37" s="14"/>
+      <c r="D37" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="H36" s="2" t="s">
+      <c r="H37" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="I36" s="19"/>
-      <c r="K36" s="13"/>
-      <c r="L36" s="6"/>
-      <c r="M36" s="8"/>
-      <c r="N36" s="8"/>
-      <c r="O36" s="8"/>
-    </row>
-    <row r="37" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B37" s="12"/>
-      <c r="D37" s="2" t="s">
+      <c r="I37" s="10"/>
+      <c r="J37" s="14"/>
+      <c r="K37" s="14"/>
+      <c r="L37" s="13"/>
+      <c r="M37" s="4"/>
+      <c r="N37" s="4"/>
+      <c r="O37" s="4"/>
+    </row>
+    <row r="38" spans="2:15" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B38" s="13"/>
+      <c r="D38" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H37" s="2" t="s">
+      <c r="E38" s="2"/>
+      <c r="F38" s="2"/>
+      <c r="G38" s="2"/>
+      <c r="H38" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="I37" s="19"/>
-      <c r="K37" s="13"/>
-      <c r="L37" s="6"/>
-      <c r="M37" s="8"/>
-      <c r="N37" s="8"/>
-      <c r="O37" s="8"/>
-    </row>
-    <row r="38" spans="2:15" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="6"/>
-      <c r="D38" s="8" t="s">
+      <c r="I38" s="10"/>
+      <c r="J38" s="14"/>
+      <c r="K38" s="13"/>
+      <c r="L38" s="13"/>
+    </row>
+    <row r="39" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B39" s="14"/>
+      <c r="D39" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="K38" s="9"/>
-      <c r="L38" s="6"/>
-    </row>
-    <row r="39" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B39" s="12"/>
-      <c r="D39" s="21"/>
-      <c r="E39" s="21"/>
-      <c r="F39" s="21"/>
-      <c r="G39" s="21"/>
-      <c r="H39" s="21"/>
-      <c r="I39" s="21"/>
-      <c r="J39" s="21"/>
-      <c r="K39" s="13"/>
-      <c r="L39" s="6"/>
-      <c r="M39" s="8"/>
-      <c r="N39" s="8"/>
-      <c r="O39" s="8"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="4"/>
+      <c r="H39" s="4"/>
+      <c r="I39" s="4"/>
+      <c r="J39" s="13"/>
+      <c r="K39" s="14"/>
+      <c r="L39" s="13"/>
+      <c r="M39" s="4"/>
+      <c r="N39" s="4"/>
+      <c r="O39" s="4"/>
     </row>
     <row r="40" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B40" s="12"/>
-      <c r="K40" s="13"/>
-      <c r="L40" s="6"/>
-      <c r="M40" s="8"/>
-      <c r="N40" s="8"/>
-      <c r="O40" s="8"/>
+      <c r="B40" s="14"/>
+      <c r="J40" s="14"/>
+      <c r="K40" s="14"/>
+      <c r="L40" s="13"/>
+      <c r="M40" s="4"/>
+      <c r="N40" s="4"/>
+      <c r="O40" s="4"/>
     </row>
     <row r="41" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B41" s="12"/>
+      <c r="B41" s="14"/>
       <c r="C41" s="2">
         <v>1</v>
       </c>
-      <c r="D41" s="8"/>
-      <c r="G41" s="8"/>
-      <c r="H41" s="8" t="s">
+      <c r="D41" s="4"/>
+      <c r="G41" s="4"/>
+      <c r="H41" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I41" s="8"/>
-      <c r="J41" s="8"/>
-      <c r="K41" s="13"/>
-      <c r="L41" s="6"/>
-      <c r="M41" s="8"/>
-      <c r="N41" s="8"/>
-      <c r="O41" s="8"/>
+      <c r="I41" s="4"/>
+      <c r="J41" s="13"/>
+      <c r="K41" s="14"/>
+      <c r="L41" s="13"/>
+      <c r="M41" s="4"/>
+      <c r="N41" s="4"/>
+      <c r="O41" s="4"/>
     </row>
     <row r="42" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B42" s="12"/>
-      <c r="K42" s="13"/>
-      <c r="L42" s="6"/>
-      <c r="M42" s="8"/>
-      <c r="N42" s="8"/>
-      <c r="O42" s="8"/>
+      <c r="B42" s="14"/>
+      <c r="J42" s="14"/>
+      <c r="K42" s="14"/>
+      <c r="L42" s="13"/>
+      <c r="M42" s="4"/>
+      <c r="N42" s="4"/>
+      <c r="O42" s="4"/>
     </row>
     <row r="43" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B43" s="12"/>
-      <c r="K43" s="13"/>
-      <c r="L43" s="6"/>
-      <c r="M43" s="8"/>
-      <c r="N43" s="8"/>
-      <c r="O43" s="8"/>
+      <c r="B43" s="14"/>
+      <c r="J43" s="14"/>
+      <c r="K43" s="14"/>
+      <c r="L43" s="13"/>
+      <c r="M43" s="4"/>
+      <c r="N43" s="4"/>
+      <c r="O43" s="4"/>
     </row>
     <row r="44" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B44" s="12"/>
-      <c r="K44" s="13"/>
-      <c r="L44" s="6"/>
-      <c r="M44" s="8"/>
-      <c r="N44" s="8"/>
-      <c r="O44" s="8"/>
+      <c r="B44" s="14"/>
+      <c r="J44" s="14"/>
+      <c r="K44" s="14"/>
+      <c r="L44" s="13"/>
+      <c r="M44" s="4"/>
+      <c r="N44" s="4"/>
+      <c r="O44" s="4"/>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B45" s="12"/>
-      <c r="K45" s="13"/>
-      <c r="L45" s="6"/>
-      <c r="M45" s="8"/>
-      <c r="N45" s="8"/>
-      <c r="O45" s="8"/>
+      <c r="B45" s="14"/>
+      <c r="J45" s="14"/>
+      <c r="K45" s="14"/>
+      <c r="L45" s="13"/>
+      <c r="M45" s="4"/>
+      <c r="N45" s="4"/>
+      <c r="O45" s="4"/>
     </row>
     <row r="46" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="12"/>
-      <c r="K46" s="13"/>
-      <c r="L46" s="6"/>
-      <c r="M46" s="8"/>
-      <c r="N46" s="8"/>
-      <c r="O46" s="8"/>
+      <c r="B46" s="14"/>
+      <c r="J46" s="14"/>
+      <c r="K46" s="14"/>
+      <c r="L46" s="13"/>
+      <c r="M46" s="4"/>
+      <c r="N46" s="4"/>
+      <c r="O46" s="4"/>
     </row>
     <row r="47" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="12"/>
-      <c r="K47" s="13"/>
-      <c r="L47" s="6"/>
-      <c r="M47" s="8"/>
-      <c r="N47" s="8"/>
-      <c r="O47" s="8"/>
+      <c r="B47" s="14"/>
+      <c r="J47" s="14"/>
+      <c r="K47" s="14"/>
+      <c r="L47" s="13"/>
+      <c r="M47" s="4"/>
+      <c r="N47" s="4"/>
+      <c r="O47" s="4"/>
     </row>
     <row r="48" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B48" s="12"/>
-      <c r="K48" s="13"/>
-      <c r="L48" s="6"/>
-      <c r="M48" s="8"/>
-      <c r="N48" s="8"/>
-      <c r="O48" s="8"/>
+      <c r="B48" s="14"/>
+      <c r="J48" s="14"/>
+      <c r="K48" s="14"/>
+      <c r="L48" s="13"/>
+      <c r="M48" s="4"/>
+      <c r="N48" s="4"/>
+      <c r="O48" s="4"/>
     </row>
     <row r="49" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B49" s="12"/>
-      <c r="K49" s="13"/>
-      <c r="L49" s="6"/>
-      <c r="M49" s="8"/>
-      <c r="N49" s="8"/>
-      <c r="O49" s="8"/>
+      <c r="B49" s="14"/>
+      <c r="J49" s="14"/>
+      <c r="K49" s="14"/>
+      <c r="L49" s="13"/>
+      <c r="M49" s="4"/>
+      <c r="N49" s="4"/>
+      <c r="O49" s="4"/>
     </row>
     <row r="50" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B50" s="12"/>
-      <c r="K50" s="13"/>
-      <c r="L50" s="6"/>
-      <c r="M50" s="8"/>
-      <c r="N50" s="8"/>
-      <c r="O50" s="8"/>
+      <c r="B50" s="14"/>
+      <c r="J50" s="14"/>
+      <c r="K50" s="14"/>
+      <c r="L50" s="13"/>
+      <c r="M50" s="4"/>
+      <c r="N50" s="4"/>
+      <c r="O50" s="4"/>
     </row>
     <row r="51" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B51" s="12"/>
-      <c r="K51" s="13"/>
-      <c r="L51" s="6"/>
-      <c r="M51" s="8"/>
-      <c r="N51" s="8"/>
-      <c r="O51" s="8"/>
+      <c r="B51" s="14"/>
+      <c r="J51" s="14"/>
+      <c r="K51" s="14"/>
+      <c r="L51" s="13"/>
+      <c r="M51" s="4"/>
+      <c r="N51" s="4"/>
+      <c r="O51" s="4"/>
     </row>
     <row r="52" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B52" s="12"/>
-      <c r="K52" s="13"/>
-      <c r="L52" s="6"/>
-      <c r="M52" s="8"/>
-      <c r="N52" s="8"/>
-      <c r="O52" s="8"/>
+      <c r="B52" s="14"/>
+      <c r="J52" s="14"/>
+      <c r="K52" s="14"/>
+      <c r="L52" s="13"/>
+      <c r="M52" s="4"/>
+      <c r="N52" s="4"/>
+      <c r="O52" s="4"/>
     </row>
     <row r="53" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B53" s="12"/>
-      <c r="K53" s="13"/>
-      <c r="L53" s="6"/>
-      <c r="M53" s="8"/>
-      <c r="N53" s="8"/>
-      <c r="O53" s="8"/>
+      <c r="B53" s="14"/>
+      <c r="J53" s="14"/>
+      <c r="K53" s="14"/>
+      <c r="L53" s="13"/>
+      <c r="M53" s="4"/>
+      <c r="N53" s="4"/>
+      <c r="O53" s="4"/>
     </row>
     <row r="54" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B54" s="12"/>
-      <c r="K54" s="13"/>
-      <c r="L54" s="6"/>
-      <c r="M54" s="8"/>
-      <c r="N54" s="8"/>
-      <c r="O54" s="8"/>
+      <c r="B54" s="14"/>
+      <c r="J54" s="14"/>
+      <c r="K54" s="14"/>
+      <c r="L54" s="13"/>
+      <c r="M54" s="4"/>
+      <c r="N54" s="4"/>
+      <c r="O54" s="4"/>
     </row>
     <row r="55" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B55" s="12"/>
-      <c r="K55" s="13"/>
-      <c r="L55" s="6"/>
-      <c r="M55" s="8"/>
-      <c r="N55" s="8"/>
-      <c r="O55" s="8"/>
+      <c r="B55" s="14"/>
+      <c r="J55" s="14"/>
+      <c r="K55" s="14"/>
+      <c r="L55" s="13"/>
+      <c r="M55" s="4"/>
+      <c r="N55" s="4"/>
+      <c r="O55" s="4"/>
     </row>
     <row r="56" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B56" s="12"/>
-      <c r="K56" s="13"/>
-      <c r="L56" s="6"/>
-      <c r="M56" s="8"/>
-      <c r="N56" s="8"/>
-      <c r="O56" s="8"/>
+      <c r="B56" s="14"/>
+      <c r="J56" s="14"/>
+      <c r="K56" s="14"/>
+      <c r="L56" s="13"/>
+      <c r="M56" s="4"/>
+      <c r="N56" s="4"/>
+      <c r="O56" s="4"/>
     </row>
     <row r="57" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B57" s="12"/>
-      <c r="K57" s="13"/>
-      <c r="L57" s="6"/>
-      <c r="M57" s="8"/>
-      <c r="N57" s="8"/>
-      <c r="O57" s="8"/>
+      <c r="B57" s="14"/>
+      <c r="J57" s="14"/>
+      <c r="K57" s="14"/>
+      <c r="L57" s="13"/>
+      <c r="M57" s="4"/>
+      <c r="N57" s="4"/>
+      <c r="O57" s="4"/>
     </row>
     <row r="58" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B58" s="12"/>
-      <c r="K58" s="13"/>
-      <c r="L58" s="6"/>
-      <c r="M58" s="8"/>
-      <c r="N58" s="8"/>
-      <c r="O58" s="8"/>
+      <c r="B58" s="14"/>
+      <c r="J58" s="14"/>
+      <c r="K58" s="14"/>
+      <c r="L58" s="13"/>
+      <c r="M58" s="4"/>
+      <c r="N58" s="4"/>
+      <c r="O58" s="4"/>
     </row>
     <row r="59" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B59" s="12"/>
-      <c r="K59" s="13"/>
-      <c r="L59" s="6"/>
-      <c r="M59" s="8"/>
-      <c r="N59" s="8"/>
-      <c r="O59" s="8"/>
+      <c r="B59" s="14"/>
+      <c r="J59" s="14"/>
+      <c r="K59" s="14"/>
+      <c r="L59" s="13"/>
+      <c r="M59" s="4"/>
+      <c r="N59" s="4"/>
+      <c r="O59" s="4"/>
     </row>
     <row r="60" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B60" s="12"/>
-      <c r="K60" s="13"/>
-      <c r="L60" s="6"/>
-      <c r="M60" s="8"/>
-      <c r="N60" s="8"/>
-      <c r="O60" s="8"/>
+      <c r="B60" s="14"/>
+      <c r="J60" s="14"/>
+      <c r="K60" s="14"/>
+      <c r="L60" s="13"/>
+      <c r="M60" s="4"/>
+      <c r="N60" s="4"/>
+      <c r="O60" s="4"/>
     </row>
     <row r="61" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B61" s="12"/>
-      <c r="K61" s="13"/>
-      <c r="L61" s="6"/>
-      <c r="M61" s="8"/>
-      <c r="N61" s="8"/>
-      <c r="O61" s="8"/>
+      <c r="B61" s="14"/>
+      <c r="J61" s="14"/>
+      <c r="K61" s="14"/>
+      <c r="L61" s="13"/>
+      <c r="M61" s="4"/>
+      <c r="N61" s="4"/>
+      <c r="O61" s="4"/>
     </row>
     <row r="62" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B62" s="12"/>
-      <c r="K62" s="13"/>
-      <c r="L62" s="6"/>
-      <c r="M62" s="8"/>
-      <c r="N62" s="8"/>
-      <c r="O62" s="8"/>
+      <c r="B62" s="14"/>
+      <c r="J62" s="14"/>
+      <c r="K62" s="14"/>
+      <c r="L62" s="13"/>
+      <c r="M62" s="4"/>
+      <c r="N62" s="4"/>
+      <c r="O62" s="4"/>
     </row>
     <row r="63" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B63" s="12"/>
-      <c r="K63" s="13"/>
-      <c r="L63" s="6"/>
-      <c r="M63" s="8"/>
-      <c r="N63" s="8"/>
-      <c r="O63" s="8"/>
+      <c r="B63" s="14"/>
+      <c r="J63" s="14"/>
+      <c r="K63" s="14"/>
+      <c r="L63" s="13"/>
+      <c r="M63" s="4"/>
+      <c r="N63" s="4"/>
+      <c r="O63" s="4"/>
     </row>
     <row r="64" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B64" s="12"/>
-      <c r="K64" s="13"/>
-      <c r="L64" s="6"/>
-      <c r="M64" s="8"/>
-      <c r="N64" s="8"/>
-      <c r="O64" s="8"/>
+      <c r="B64" s="14"/>
+      <c r="J64" s="14"/>
+      <c r="K64" s="14"/>
+      <c r="L64" s="13"/>
+      <c r="M64" s="4"/>
+      <c r="N64" s="4"/>
+      <c r="O64" s="4"/>
     </row>
     <row r="65" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B65" s="12"/>
-      <c r="K65" s="13"/>
-      <c r="L65" s="6"/>
-      <c r="M65" s="8"/>
-      <c r="N65" s="8"/>
-      <c r="O65" s="8"/>
+      <c r="B65" s="14"/>
+      <c r="J65" s="14"/>
+      <c r="K65" s="14"/>
+      <c r="L65" s="13"/>
+      <c r="M65" s="4"/>
+      <c r="N65" s="4"/>
+      <c r="O65" s="4"/>
     </row>
     <row r="66" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B66" s="12"/>
-      <c r="K66" s="13"/>
-      <c r="L66" s="6"/>
-      <c r="M66" s="8"/>
-      <c r="N66" s="8"/>
-      <c r="O66" s="8"/>
+      <c r="B66" s="14"/>
+      <c r="J66" s="14"/>
+      <c r="K66" s="14"/>
+      <c r="L66" s="13"/>
+      <c r="M66" s="4"/>
+      <c r="N66" s="4"/>
+      <c r="O66" s="4"/>
     </row>
     <row r="67" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B67" s="12"/>
-      <c r="K67" s="13"/>
-      <c r="L67" s="6"/>
-      <c r="M67" s="8"/>
-      <c r="N67" s="8"/>
-      <c r="O67" s="8"/>
+      <c r="B67" s="14"/>
+      <c r="J67" s="14"/>
+      <c r="K67" s="14"/>
+      <c r="L67" s="13"/>
+      <c r="M67" s="4"/>
+      <c r="N67" s="4"/>
+      <c r="O67" s="4"/>
     </row>
     <row r="68" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B68" s="12"/>
-      <c r="K68" s="13"/>
-      <c r="L68" s="6"/>
-      <c r="M68" s="8"/>
-      <c r="N68" s="8"/>
-      <c r="O68" s="8"/>
+      <c r="B68" s="14"/>
+      <c r="J68" s="14"/>
+      <c r="K68" s="14"/>
+      <c r="L68" s="13"/>
+      <c r="M68" s="4"/>
+      <c r="N68" s="4"/>
+      <c r="O68" s="4"/>
     </row>
     <row r="69" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B69" s="12"/>
-      <c r="K69" s="13"/>
-      <c r="L69" s="6"/>
-      <c r="M69" s="8"/>
-      <c r="N69" s="8"/>
-      <c r="O69" s="8"/>
+      <c r="B69" s="14"/>
+      <c r="J69" s="14"/>
+      <c r="K69" s="14"/>
+      <c r="L69" s="13"/>
+      <c r="M69" s="4"/>
+      <c r="N69" s="4"/>
+      <c r="O69" s="4"/>
     </row>
     <row r="70" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B70" s="12"/>
-      <c r="K70" s="13"/>
-      <c r="L70" s="6"/>
-      <c r="M70" s="8"/>
-      <c r="N70" s="8"/>
-      <c r="O70" s="8"/>
+      <c r="B70" s="14"/>
+      <c r="J70" s="14"/>
+      <c r="K70" s="14"/>
+      <c r="L70" s="13"/>
+      <c r="M70" s="4"/>
+      <c r="N70" s="4"/>
+      <c r="O70" s="4"/>
     </row>
     <row r="71" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B71" s="12"/>
-      <c r="K71" s="13"/>
-      <c r="L71" s="6"/>
-      <c r="M71" s="8"/>
-      <c r="N71" s="8"/>
-      <c r="O71" s="8"/>
+      <c r="B71" s="14"/>
+      <c r="J71" s="14"/>
+      <c r="K71" s="14"/>
+      <c r="L71" s="13"/>
+      <c r="M71" s="4"/>
+      <c r="N71" s="4"/>
+      <c r="O71" s="4"/>
     </row>
     <row r="72" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B72" s="12"/>
-      <c r="K72" s="13"/>
-      <c r="L72" s="6"/>
-      <c r="M72" s="8"/>
-      <c r="N72" s="8"/>
-      <c r="O72" s="8"/>
+      <c r="B72" s="14"/>
+      <c r="J72" s="14"/>
+      <c r="K72" s="14"/>
+      <c r="L72" s="13"/>
+      <c r="M72" s="4"/>
+      <c r="N72" s="4"/>
+      <c r="O72" s="4"/>
     </row>
     <row r="73" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B73" s="12"/>
-      <c r="K73" s="13"/>
-      <c r="L73" s="6"/>
-      <c r="M73" s="8"/>
-      <c r="N73" s="8"/>
-      <c r="O73" s="8"/>
+      <c r="B73" s="14"/>
+      <c r="J73" s="14"/>
+      <c r="K73" s="14"/>
+      <c r="L73" s="13"/>
+      <c r="M73" s="4"/>
+      <c r="N73" s="4"/>
+      <c r="O73" s="4"/>
     </row>
     <row r="74" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B74" s="12"/>
-      <c r="K74" s="13"/>
-      <c r="L74" s="6"/>
-      <c r="M74" s="8"/>
-      <c r="N74" s="8"/>
-      <c r="O74" s="8"/>
+      <c r="B74" s="14"/>
+      <c r="J74" s="14"/>
+      <c r="K74" s="14"/>
+      <c r="L74" s="13"/>
+      <c r="M74" s="4"/>
+      <c r="N74" s="4"/>
+      <c r="O74" s="4"/>
     </row>
     <row r="75" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B75" s="12"/>
-      <c r="K75" s="13"/>
-      <c r="L75" s="6"/>
-      <c r="M75" s="8"/>
-      <c r="N75" s="8"/>
-      <c r="O75" s="8"/>
+      <c r="B75" s="14"/>
+      <c r="J75" s="14"/>
+      <c r="K75" s="14"/>
+      <c r="L75" s="13"/>
+      <c r="M75" s="4"/>
+      <c r="N75" s="4"/>
+      <c r="O75" s="4"/>
     </row>
     <row r="76" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B76" s="12"/>
-      <c r="K76" s="13"/>
-      <c r="L76" s="6"/>
-      <c r="M76" s="8"/>
-      <c r="N76" s="8"/>
-      <c r="O76" s="8"/>
+      <c r="B76" s="14"/>
+      <c r="J76" s="14"/>
+      <c r="K76" s="14"/>
+      <c r="L76" s="13"/>
+      <c r="M76" s="4"/>
+      <c r="N76" s="4"/>
+      <c r="O76" s="4"/>
     </row>
     <row r="77" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B77" s="12"/>
-      <c r="K77" s="13"/>
-      <c r="L77" s="17"/>
+      <c r="B77" s="14"/>
+      <c r="J77" s="14"/>
+      <c r="K77" s="14"/>
+      <c r="L77" s="12"/>
     </row>
     <row r="78" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B78" s="12"/>
-      <c r="H78" s="8"/>
-      <c r="I78" s="8"/>
-      <c r="J78" s="8"/>
-      <c r="K78" s="13"/>
+      <c r="B78" s="14"/>
+      <c r="H78" s="4"/>
+      <c r="I78" s="4"/>
+      <c r="J78" s="13"/>
+      <c r="K78" s="14"/>
     </row>
     <row r="79" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B79" s="12"/>
-      <c r="K79" s="13"/>
+      <c r="B79" s="14"/>
+      <c r="J79" s="14"/>
+      <c r="K79" s="14"/>
     </row>
     <row r="80" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B80" s="12"/>
-      <c r="K80" s="13"/>
+      <c r="B80" s="14"/>
+      <c r="J80" s="14"/>
+      <c r="K80" s="14"/>
     </row>
     <row r="81" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B81" s="12"/>
-      <c r="K81" s="13"/>
+      <c r="B81" s="14"/>
+      <c r="J81" s="14"/>
+      <c r="K81" s="14"/>
     </row>
     <row r="82" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B82" s="12"/>
-      <c r="K82" s="13"/>
+      <c r="B82" s="14"/>
+      <c r="J82" s="14"/>
+      <c r="K82" s="14"/>
     </row>
     <row r="83" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B83" s="12"/>
-      <c r="K83" s="13"/>
+      <c r="B83" s="14"/>
+      <c r="J83" s="14"/>
+      <c r="K83" s="14"/>
     </row>
     <row r="84" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B84" s="12"/>
-      <c r="K84" s="13"/>
+      <c r="B84" s="14"/>
+      <c r="J84" s="14"/>
+      <c r="K84" s="14"/>
     </row>
     <row r="85" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B85" s="12"/>
-      <c r="K85" s="13"/>
+      <c r="B85" s="14"/>
+      <c r="J85" s="14"/>
+      <c r="K85" s="14"/>
     </row>
     <row r="86" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B86" s="12"/>
-      <c r="K86" s="13"/>
+      <c r="B86" s="14"/>
+      <c r="J86" s="14"/>
+      <c r="K86" s="14"/>
     </row>
     <row r="87" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B87" s="12"/>
-      <c r="K87" s="13"/>
+      <c r="B87" s="14"/>
+      <c r="J87" s="14"/>
+      <c r="K87" s="14"/>
     </row>
     <row r="88" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B88" s="12"/>
-      <c r="K88" s="13"/>
+      <c r="B88" s="14"/>
+      <c r="J88" s="14"/>
+      <c r="K88" s="14"/>
     </row>
     <row r="89" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B89" s="12"/>
-      <c r="K89" s="13"/>
+      <c r="B89" s="14"/>
+      <c r="J89" s="14"/>
+      <c r="K89" s="14"/>
     </row>
     <row r="90" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B90" s="12"/>
-      <c r="K90" s="13"/>
+      <c r="B90" s="14"/>
+      <c r="J90" s="14"/>
+      <c r="K90" s="14"/>
     </row>
     <row r="91" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B91" s="12"/>
-      <c r="K91" s="13"/>
+      <c r="B91" s="14"/>
+      <c r="J91" s="14"/>
+      <c r="K91" s="14"/>
     </row>
     <row r="92" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B92" s="12"/>
-      <c r="K92" s="13"/>
+      <c r="B92" s="14"/>
+      <c r="J92" s="14"/>
+      <c r="K92" s="14"/>
     </row>
     <row r="93" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B93" s="12"/>
-      <c r="K93" s="13"/>
+      <c r="B93" s="14"/>
+      <c r="J93" s="14"/>
+      <c r="K93" s="14"/>
     </row>
     <row r="94" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B94" s="12"/>
-      <c r="K94" s="13"/>
+      <c r="B94" s="14"/>
+      <c r="J94" s="14"/>
+      <c r="K94" s="14"/>
     </row>
     <row r="95" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B95" s="12"/>
-      <c r="K95" s="13"/>
+      <c r="B95" s="14"/>
+      <c r="J95" s="14"/>
+      <c r="K95" s="14"/>
     </row>
     <row r="96" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B96" s="12"/>
-      <c r="K96" s="13"/>
+      <c r="B96" s="14"/>
+      <c r="J96" s="14"/>
+      <c r="K96" s="14"/>
     </row>
     <row r="97" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B97" s="12"/>
-      <c r="K97" s="13"/>
+      <c r="B97" s="14"/>
+      <c r="J97" s="14"/>
+      <c r="K97" s="14"/>
     </row>
     <row r="98" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B98" s="12"/>
-      <c r="K98" s="13"/>
+      <c r="B98" s="14"/>
+      <c r="J98" s="14"/>
+      <c r="K98" s="14"/>
     </row>
     <row r="99" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B99" s="12"/>
-      <c r="K99" s="13"/>
+      <c r="B99" s="14"/>
+      <c r="J99" s="14"/>
+      <c r="K99" s="14"/>
     </row>
     <row r="100" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B100" s="12"/>
-      <c r="K100" s="13"/>
+      <c r="B100" s="14"/>
+      <c r="J100" s="14"/>
+      <c r="K100" s="14"/>
+    </row>
+    <row r="101" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B101" s="14"/>
+      <c r="J101" s="14"/>
+      <c r="K101" s="14"/>
+    </row>
+    <row r="102" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B102" s="14"/>
+      <c r="J102" s="14"/>
+      <c r="K102" s="14"/>
+    </row>
+    <row r="103" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B103" s="14"/>
+    </row>
+    <row r="104" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B104" s="14"/>
+    </row>
+    <row r="105" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B105" s="14"/>
+    </row>
+    <row r="106" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B106" s="14"/>
+    </row>
+    <row r="107" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B107" s="14"/>
+    </row>
+    <row r="108" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B108" s="14"/>
+    </row>
+    <row r="109" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B109" s="14"/>
+    </row>
+    <row r="110" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B110" s="14"/>
+    </row>
+    <row r="111" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B111" s="14"/>
+    </row>
+    <row r="112" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B112" s="14"/>
+    </row>
+    <row r="113" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B113" s="14"/>
+    </row>
+    <row r="114" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B114" s="14"/>
+    </row>
+    <row r="115" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B115" s="14"/>
+    </row>
+    <row r="116" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B116" s="14"/>
+    </row>
+    <row r="117" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B117" s="14"/>
+    </row>
+    <row r="118" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B118" s="14"/>
+    </row>
+    <row r="119" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B119" s="14"/>
+    </row>
+    <row r="120" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B120" s="14"/>
+    </row>
+    <row r="121" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B121" s="14"/>
+    </row>
+    <row r="122" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B122" s="14"/>
+    </row>
+    <row r="123" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B123" s="14"/>
+    </row>
+    <row r="124" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B124" s="14"/>
+    </row>
+    <row r="125" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B125" s="14"/>
+    </row>
+    <row r="126" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B126" s="14"/>
+    </row>
+    <row r="127" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B127" s="14"/>
+    </row>
+    <row r="128" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B128" s="14"/>
+    </row>
+    <row r="129" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B129" s="14"/>
+    </row>
+    <row r="130" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B130" s="14"/>
+    </row>
+    <row r="131" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B131" s="14"/>
+    </row>
+    <row r="132" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B132" s="14"/>
+    </row>
+    <row r="133" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B133" s="14"/>
+    </row>
+    <row r="134" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B134" s="14"/>
+    </row>
+    <row r="135" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B135" s="14"/>
+    </row>
+    <row r="136" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B136" s="14"/>
+    </row>
+    <row r="137" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B137" s="14"/>
+    </row>
+    <row r="138" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B138" s="14"/>
+    </row>
+    <row r="139" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B139" s="14"/>
+    </row>
+    <row r="140" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B140" s="14"/>
+    </row>
+    <row r="141" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B141" s="14"/>
+    </row>
+    <row r="142" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B142" s="14"/>
+    </row>
+    <row r="143" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B143" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="D39:J39"/>
-  </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="8" scale="49" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="57" fitToHeight="72" orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;A</oddHeader>
+    <oddFooter>Page &amp;P of &amp;N</oddFooter>
+  </headerFooter>
+  <rowBreaks count="2" manualBreakCount="2">
+    <brk id="41" max="11" man="1"/>
+    <brk id="75" max="11" man="1"/>
+  </rowBreaks>
+  <colBreaks count="1" manualBreakCount="1">
+    <brk id="3" max="149" man="1"/>
+  </colBreaks>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
@@ -7123,25 +7270,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="11" t="s">
         <v>23</v>
       </c>
       <c r="B1" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="11" t="s">
         <v>22</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="11" t="s">
         <v>24</v>
       </c>
       <c r="F1" t="s">
         <v>26</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="G1" s="11" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
server Worker: StartPeriodicRunningTestUpdate - update state (BPT query message), update pdf template
</commit_message>
<xml_diff>
--- a/web-console/server/assets/pdf_template.xlsx
+++ b/web-console/server/assets/pdf_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\DEV\UBA6\web-console\server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9405F6C-6F14-491E-8CB2-E88E31A50346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FDEBAEB-E12F-4A4F-92EF-492B61E60570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
   </bookViews>
@@ -218,7 +218,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
@@ -241,14 +241,6 @@
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6123,7 +6115,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:O143"/>
+  <dimension ref="B2:O78"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.44140625" style="2" customWidth="1"/>
@@ -6139,30 +6131,11 @@
     <col min="16" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-    </row>
     <row r="2" spans="2:14" ht="8.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="13"/>
-      <c r="K2" s="14"/>
+      <c r="J2" s="4"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B3" s="13"/>
+      <c r="B3" s="4"/>
       <c r="D3" s="3" t="s">
         <v>16</v>
       </c>
@@ -6173,14 +6146,14 @@
       <c r="H3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="J3" s="13" t="s">
+      <c r="J3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="K3" s="13"/>
+      <c r="K3" s="4"/>
       <c r="N3" s="5"/>
     </row>
     <row r="4" spans="2:14" ht="5.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="13"/>
+      <c r="B4" s="4"/>
       <c r="C4" s="6"/>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -6188,12 +6161,11 @@
       <c r="G4" s="6"/>
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
-      <c r="J4" s="13"/>
-      <c r="K4" s="13"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
       <c r="N4" s="5"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B5" s="14"/>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
@@ -6201,11 +6173,9 @@
       <c r="G5" s="9"/>
       <c r="H5" s="9"/>
       <c r="I5" s="9"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="14"/>
+      <c r="J5" s="9"/>
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B6" s="14"/>
       <c r="C6" s="9"/>
       <c r="D6" s="9"/>
       <c r="E6" s="9"/>
@@ -6213,11 +6183,9 @@
       <c r="G6" s="9"/>
       <c r="H6" s="9"/>
       <c r="I6" s="9"/>
-      <c r="J6" s="15"/>
-      <c r="K6" s="14"/>
+      <c r="J6" s="9"/>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B7" s="14"/>
       <c r="C7" s="9"/>
       <c r="D7" s="9"/>
       <c r="E7" s="9"/>
@@ -6225,11 +6193,9 @@
       <c r="G7" s="9"/>
       <c r="H7" s="9"/>
       <c r="I7" s="9"/>
-      <c r="J7" s="15"/>
-      <c r="K7" s="14"/>
+      <c r="J7" s="9"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B8" s="14"/>
       <c r="C8" s="9"/>
       <c r="D8" s="9"/>
       <c r="E8" s="9"/>
@@ -6237,11 +6203,9 @@
       <c r="G8" s="9"/>
       <c r="H8" s="9"/>
       <c r="I8" s="9"/>
-      <c r="J8" s="15"/>
-      <c r="K8" s="14"/>
+      <c r="J8" s="9"/>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B9" s="14"/>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
@@ -6249,11 +6213,9 @@
       <c r="G9" s="9"/>
       <c r="H9" s="9"/>
       <c r="I9" s="9"/>
-      <c r="J9" s="15"/>
-      <c r="K9" s="14"/>
+      <c r="J9" s="9"/>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B10" s="14"/>
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
@@ -6261,11 +6223,9 @@
       <c r="G10" s="9"/>
       <c r="H10" s="9"/>
       <c r="I10" s="9"/>
-      <c r="J10" s="15"/>
-      <c r="K10" s="14"/>
+      <c r="J10" s="9"/>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B11" s="14"/>
       <c r="C11" s="9"/>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
@@ -6273,11 +6233,9 @@
       <c r="G11" s="9"/>
       <c r="H11" s="9"/>
       <c r="I11" s="9"/>
-      <c r="J11" s="15"/>
-      <c r="K11" s="14"/>
+      <c r="J11" s="9"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B12" s="14"/>
       <c r="C12" s="9"/>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
@@ -6285,11 +6243,9 @@
       <c r="G12" s="9"/>
       <c r="H12" s="9"/>
       <c r="I12" s="9"/>
-      <c r="J12" s="15"/>
-      <c r="K12" s="14"/>
+      <c r="J12" s="9"/>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B13" s="14"/>
       <c r="C13" s="9"/>
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
@@ -6297,11 +6253,9 @@
       <c r="G13" s="9"/>
       <c r="H13" s="9"/>
       <c r="I13" s="9"/>
-      <c r="J13" s="15"/>
-      <c r="K13" s="14"/>
+      <c r="J13" s="9"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B14" s="14"/>
       <c r="C14" s="9"/>
       <c r="D14" s="9"/>
       <c r="E14" s="9"/>
@@ -6309,11 +6263,9 @@
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
       <c r="I14" s="9"/>
-      <c r="J14" s="15"/>
-      <c r="K14" s="14"/>
+      <c r="J14" s="9"/>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B15" s="14"/>
       <c r="C15" s="9"/>
       <c r="D15" s="9"/>
       <c r="E15" s="9"/>
@@ -6321,11 +6273,9 @@
       <c r="G15" s="9"/>
       <c r="H15" s="9"/>
       <c r="I15" s="9"/>
-      <c r="J15" s="15"/>
-      <c r="K15" s="14"/>
+      <c r="J15" s="9"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B16" s="14"/>
       <c r="C16" s="9"/>
       <c r="D16" s="9"/>
       <c r="E16" s="9"/>
@@ -6333,11 +6283,9 @@
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
       <c r="I16" s="9"/>
-      <c r="J16" s="15"/>
-      <c r="K16" s="14"/>
+      <c r="J16" s="9"/>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B17" s="14"/>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
@@ -6345,11 +6293,9 @@
       <c r="G17" s="9"/>
       <c r="H17" s="9"/>
       <c r="I17" s="9"/>
-      <c r="J17" s="15"/>
-      <c r="K17" s="14"/>
+      <c r="J17" s="9"/>
     </row>
     <row r="18" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B18" s="14"/>
       <c r="C18" s="9"/>
       <c r="D18" s="9"/>
       <c r="E18" s="9"/>
@@ -6357,11 +6303,9 @@
       <c r="G18" s="9"/>
       <c r="H18" s="9"/>
       <c r="I18" s="9"/>
-      <c r="J18" s="15"/>
-      <c r="K18" s="14"/>
+      <c r="J18" s="9"/>
     </row>
     <row r="19" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B19" s="14"/>
       <c r="C19" s="9"/>
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
@@ -6369,11 +6313,9 @@
       <c r="G19" s="9"/>
       <c r="H19" s="9"/>
       <c r="I19" s="9"/>
-      <c r="J19" s="15"/>
-      <c r="K19" s="14"/>
+      <c r="J19" s="9"/>
     </row>
     <row r="20" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B20" s="14"/>
       <c r="C20" s="9"/>
       <c r="D20" s="9"/>
       <c r="E20" s="9"/>
@@ -6381,11 +6323,9 @@
       <c r="G20" s="9"/>
       <c r="H20" s="9"/>
       <c r="I20" s="9"/>
-      <c r="J20" s="15"/>
-      <c r="K20" s="14"/>
+      <c r="J20" s="9"/>
     </row>
     <row r="21" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B21" s="14"/>
       <c r="C21" s="9"/>
       <c r="D21" s="9"/>
       <c r="E21" s="9"/>
@@ -6393,11 +6333,9 @@
       <c r="G21" s="9"/>
       <c r="H21" s="9"/>
       <c r="I21" s="9"/>
-      <c r="J21" s="15"/>
-      <c r="K21" s="14"/>
+      <c r="J21" s="9"/>
     </row>
     <row r="22" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B22" s="14"/>
       <c r="C22" s="9"/>
       <c r="D22" s="9"/>
       <c r="E22" s="9"/>
@@ -6405,11 +6343,9 @@
       <c r="G22" s="9"/>
       <c r="H22" s="9"/>
       <c r="I22" s="9"/>
-      <c r="J22" s="15"/>
-      <c r="K22" s="14"/>
+      <c r="J22" s="9"/>
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B23" s="14"/>
       <c r="C23" s="9"/>
       <c r="D23" s="9"/>
       <c r="E23" s="9"/>
@@ -6417,11 +6353,9 @@
       <c r="G23" s="9"/>
       <c r="H23" s="9"/>
       <c r="I23" s="9"/>
-      <c r="J23" s="15"/>
-      <c r="K23" s="14"/>
+      <c r="J23" s="9"/>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B24" s="14"/>
       <c r="C24" s="9"/>
       <c r="D24" s="9"/>
       <c r="E24" s="9"/>
@@ -6429,11 +6363,9 @@
       <c r="G24" s="9"/>
       <c r="H24" s="9"/>
       <c r="I24" s="9"/>
-      <c r="J24" s="15"/>
-      <c r="K24" s="14"/>
+      <c r="J24" s="9"/>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B25" s="14"/>
       <c r="C25" s="9"/>
       <c r="D25" s="9"/>
       <c r="E25" s="9"/>
@@ -6441,11 +6373,9 @@
       <c r="G25" s="9"/>
       <c r="H25" s="9"/>
       <c r="I25" s="9"/>
-      <c r="J25" s="15"/>
-      <c r="K25" s="14"/>
+      <c r="J25" s="9"/>
     </row>
     <row r="26" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B26" s="14"/>
       <c r="C26" s="9"/>
       <c r="D26" s="9"/>
       <c r="E26" s="9"/>
@@ -6453,23 +6383,14 @@
       <c r="G26" s="9"/>
       <c r="H26" s="9"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="15"/>
-      <c r="K26" s="14"/>
+      <c r="J26" s="9"/>
       <c r="M26" s="7"/>
     </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B27" s="14"/>
-      <c r="J27" s="14"/>
-      <c r="K27" s="14"/>
-    </row>
     <row r="28" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B28" s="13"/>
-      <c r="J28" s="14"/>
-      <c r="K28" s="13"/>
-      <c r="L28" s="12"/>
+      <c r="B28" s="4"/>
+      <c r="K28" s="4"/>
     </row>
     <row r="29" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B29" s="14"/>
       <c r="D29" s="4" t="s">
         <v>15</v>
       </c>
@@ -6480,12 +6401,9 @@
         <v>14</v>
       </c>
       <c r="I29" s="4"/>
-      <c r="J29" s="13"/>
-      <c r="K29" s="14"/>
-      <c r="L29" s="12"/>
+      <c r="J29" s="4"/>
     </row>
     <row r="30" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B30" s="14"/>
       <c r="D30" s="2" t="s">
         <v>13</v>
       </c>
@@ -6493,28 +6411,22 @@
         <v>18</v>
       </c>
       <c r="I30" s="10"/>
-      <c r="J30" s="14"/>
-      <c r="K30" s="14"/>
-      <c r="L30" s="13"/>
+      <c r="L30" s="4"/>
       <c r="M30" s="4"/>
       <c r="N30" s="4"/>
       <c r="O30" s="4"/>
     </row>
     <row r="31" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B31" s="14"/>
       <c r="H31" s="2" t="s">
         <v>19</v>
       </c>
       <c r="I31" s="10"/>
-      <c r="J31" s="14"/>
-      <c r="K31" s="14"/>
-      <c r="L31" s="13"/>
+      <c r="L31" s="4"/>
       <c r="M31" s="4"/>
       <c r="N31" s="4"/>
       <c r="O31" s="4"/>
     </row>
     <row r="32" spans="2:15" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="13"/>
       <c r="D32" s="2" t="s">
         <v>12</v>
       </c>
@@ -6525,12 +6437,9 @@
         <v>11</v>
       </c>
       <c r="I32" s="10"/>
-      <c r="J32" s="14"/>
-      <c r="K32" s="13"/>
-      <c r="L32" s="13"/>
-    </row>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B33" s="14"/>
+      <c r="J32" s="2"/>
+    </row>
+    <row r="33" spans="3:15" x14ac:dyDescent="0.3">
       <c r="D33" s="2" t="s">
         <v>10</v>
       </c>
@@ -6538,60 +6447,51 @@
         <v>20</v>
       </c>
       <c r="I33" s="10"/>
-      <c r="J33" s="14" t="s">
+      <c r="J33" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="K33" s="14"/>
-      <c r="L33" s="13"/>
+      <c r="L33" s="4"/>
       <c r="M33" s="4"/>
       <c r="N33" s="4"/>
       <c r="O33" s="4"/>
     </row>
-    <row r="34" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B34" s="14"/>
+    <row r="34" spans="3:15" x14ac:dyDescent="0.3">
       <c r="H34" s="2" t="s">
         <v>21</v>
       </c>
       <c r="I34" s="10"/>
-      <c r="J34" s="14" t="s">
+      <c r="J34" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="K34" s="14"/>
-      <c r="L34" s="13"/>
+      <c r="L34" s="4"/>
       <c r="M34" s="4"/>
       <c r="N34" s="4"/>
       <c r="O34" s="4"/>
     </row>
-    <row r="35" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B35" s="14"/>
+    <row r="35" spans="3:15" x14ac:dyDescent="0.3">
       <c r="H35" s="2" t="s">
         <v>9</v>
       </c>
       <c r="I35" s="10"/>
-      <c r="J35" s="14" t="s">
+      <c r="J35" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="K35" s="14"/>
-      <c r="L35" s="13"/>
+      <c r="L35" s="4"/>
       <c r="M35" s="4"/>
       <c r="N35" s="4"/>
       <c r="O35" s="4"/>
     </row>
-    <row r="36" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B36" s="14"/>
+    <row r="36" spans="3:15" x14ac:dyDescent="0.3">
       <c r="H36" s="2" t="s">
         <v>7</v>
       </c>
       <c r="I36" s="10"/>
-      <c r="J36" s="14"/>
-      <c r="K36" s="14"/>
-      <c r="L36" s="13"/>
+      <c r="L36" s="4"/>
       <c r="M36" s="4"/>
       <c r="N36" s="4"/>
       <c r="O36" s="4"/>
     </row>
-    <row r="37" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B37" s="14"/>
+    <row r="37" spans="3:15" x14ac:dyDescent="0.3">
       <c r="D37" s="2" t="s">
         <v>8</v>
       </c>
@@ -6599,15 +6499,12 @@
         <v>5</v>
       </c>
       <c r="I37" s="10"/>
-      <c r="J37" s="14"/>
-      <c r="K37" s="14"/>
-      <c r="L37" s="13"/>
+      <c r="L37" s="4"/>
       <c r="M37" s="4"/>
       <c r="N37" s="4"/>
       <c r="O37" s="4"/>
     </row>
-    <row r="38" spans="2:15" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="13"/>
+    <row r="38" spans="3:15" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="D38" s="2" t="s">
         <v>6</v>
       </c>
@@ -6618,12 +6515,9 @@
         <v>4</v>
       </c>
       <c r="I38" s="10"/>
-      <c r="J38" s="14"/>
-      <c r="K38" s="13"/>
-      <c r="L38" s="13"/>
-    </row>
-    <row r="39" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B39" s="14"/>
+      <c r="J38" s="2"/>
+    </row>
+    <row r="39" spans="3:15" x14ac:dyDescent="0.3">
       <c r="D39" s="4" t="s">
         <v>3</v>
       </c>
@@ -6632,24 +6526,19 @@
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
       <c r="I39" s="4"/>
-      <c r="J39" s="13"/>
-      <c r="K39" s="14"/>
-      <c r="L39" s="13"/>
+      <c r="J39" s="4"/>
+      <c r="L39" s="4"/>
       <c r="M39" s="4"/>
       <c r="N39" s="4"/>
       <c r="O39" s="4"/>
     </row>
-    <row r="40" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B40" s="14"/>
-      <c r="J40" s="14"/>
-      <c r="K40" s="14"/>
-      <c r="L40" s="13"/>
+    <row r="40" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="L40" s="4"/>
       <c r="M40" s="4"/>
       <c r="N40" s="4"/>
       <c r="O40" s="4"/>
     </row>
-    <row r="41" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B41" s="14"/>
+    <row r="41" spans="3:15" x14ac:dyDescent="0.3">
       <c r="C41" s="2">
         <v>1</v>
       </c>
@@ -6659,589 +6548,232 @@
         <v>2</v>
       </c>
       <c r="I41" s="4"/>
-      <c r="J41" s="13"/>
-      <c r="K41" s="14"/>
-      <c r="L41" s="13"/>
+      <c r="J41" s="4"/>
+      <c r="L41" s="4"/>
       <c r="M41" s="4"/>
       <c r="N41" s="4"/>
       <c r="O41" s="4"/>
     </row>
-    <row r="42" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B42" s="14"/>
-      <c r="J42" s="14"/>
-      <c r="K42" s="14"/>
-      <c r="L42" s="13"/>
+    <row r="42" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="L42" s="4"/>
       <c r="M42" s="4"/>
       <c r="N42" s="4"/>
       <c r="O42" s="4"/>
     </row>
-    <row r="43" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B43" s="14"/>
-      <c r="J43" s="14"/>
-      <c r="K43" s="14"/>
-      <c r="L43" s="13"/>
+    <row r="43" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="L43" s="4"/>
       <c r="M43" s="4"/>
       <c r="N43" s="4"/>
       <c r="O43" s="4"/>
     </row>
-    <row r="44" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B44" s="14"/>
-      <c r="J44" s="14"/>
-      <c r="K44" s="14"/>
-      <c r="L44" s="13"/>
+    <row r="44" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="L44" s="4"/>
       <c r="M44" s="4"/>
       <c r="N44" s="4"/>
       <c r="O44" s="4"/>
     </row>
-    <row r="45" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B45" s="14"/>
-      <c r="J45" s="14"/>
-      <c r="K45" s="14"/>
-      <c r="L45" s="13"/>
+    <row r="45" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="L45" s="4"/>
       <c r="M45" s="4"/>
       <c r="N45" s="4"/>
       <c r="O45" s="4"/>
     </row>
-    <row r="46" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="14"/>
-      <c r="J46" s="14"/>
-      <c r="K46" s="14"/>
-      <c r="L46" s="13"/>
+    <row r="46" spans="3:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L46" s="4"/>
       <c r="M46" s="4"/>
       <c r="N46" s="4"/>
       <c r="O46" s="4"/>
     </row>
-    <row r="47" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="14"/>
-      <c r="J47" s="14"/>
-      <c r="K47" s="14"/>
-      <c r="L47" s="13"/>
+    <row r="47" spans="3:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L47" s="4"/>
       <c r="M47" s="4"/>
       <c r="N47" s="4"/>
       <c r="O47" s="4"/>
     </row>
-    <row r="48" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B48" s="14"/>
-      <c r="J48" s="14"/>
-      <c r="K48" s="14"/>
-      <c r="L48" s="13"/>
+    <row r="48" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="L48" s="4"/>
       <c r="M48" s="4"/>
       <c r="N48" s="4"/>
       <c r="O48" s="4"/>
     </row>
-    <row r="49" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B49" s="14"/>
-      <c r="J49" s="14"/>
-      <c r="K49" s="14"/>
-      <c r="L49" s="13"/>
+    <row r="49" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L49" s="4"/>
       <c r="M49" s="4"/>
       <c r="N49" s="4"/>
       <c r="O49" s="4"/>
     </row>
-    <row r="50" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B50" s="14"/>
-      <c r="J50" s="14"/>
-      <c r="K50" s="14"/>
-      <c r="L50" s="13"/>
+    <row r="50" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L50" s="4"/>
       <c r="M50" s="4"/>
       <c r="N50" s="4"/>
       <c r="O50" s="4"/>
     </row>
-    <row r="51" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B51" s="14"/>
-      <c r="J51" s="14"/>
-      <c r="K51" s="14"/>
-      <c r="L51" s="13"/>
+    <row r="51" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L51" s="4"/>
       <c r="M51" s="4"/>
       <c r="N51" s="4"/>
       <c r="O51" s="4"/>
     </row>
-    <row r="52" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B52" s="14"/>
-      <c r="J52" s="14"/>
-      <c r="K52" s="14"/>
-      <c r="L52" s="13"/>
+    <row r="52" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L52" s="4"/>
       <c r="M52" s="4"/>
       <c r="N52" s="4"/>
       <c r="O52" s="4"/>
     </row>
-    <row r="53" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B53" s="14"/>
-      <c r="J53" s="14"/>
-      <c r="K53" s="14"/>
-      <c r="L53" s="13"/>
+    <row r="53" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L53" s="4"/>
       <c r="M53" s="4"/>
       <c r="N53" s="4"/>
       <c r="O53" s="4"/>
     </row>
-    <row r="54" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B54" s="14"/>
-      <c r="J54" s="14"/>
-      <c r="K54" s="14"/>
-      <c r="L54" s="13"/>
+    <row r="54" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L54" s="4"/>
       <c r="M54" s="4"/>
       <c r="N54" s="4"/>
       <c r="O54" s="4"/>
     </row>
-    <row r="55" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B55" s="14"/>
-      <c r="J55" s="14"/>
-      <c r="K55" s="14"/>
-      <c r="L55" s="13"/>
+    <row r="55" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L55" s="4"/>
       <c r="M55" s="4"/>
       <c r="N55" s="4"/>
       <c r="O55" s="4"/>
     </row>
-    <row r="56" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B56" s="14"/>
-      <c r="J56" s="14"/>
-      <c r="K56" s="14"/>
-      <c r="L56" s="13"/>
+    <row r="56" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L56" s="4"/>
       <c r="M56" s="4"/>
       <c r="N56" s="4"/>
       <c r="O56" s="4"/>
     </row>
-    <row r="57" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B57" s="14"/>
-      <c r="J57" s="14"/>
-      <c r="K57" s="14"/>
-      <c r="L57" s="13"/>
+    <row r="57" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L57" s="4"/>
       <c r="M57" s="4"/>
       <c r="N57" s="4"/>
       <c r="O57" s="4"/>
     </row>
-    <row r="58" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B58" s="14"/>
-      <c r="J58" s="14"/>
-      <c r="K58" s="14"/>
-      <c r="L58" s="13"/>
+    <row r="58" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L58" s="4"/>
       <c r="M58" s="4"/>
       <c r="N58" s="4"/>
       <c r="O58" s="4"/>
     </row>
-    <row r="59" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B59" s="14"/>
-      <c r="J59" s="14"/>
-      <c r="K59" s="14"/>
-      <c r="L59" s="13"/>
+    <row r="59" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L59" s="4"/>
       <c r="M59" s="4"/>
       <c r="N59" s="4"/>
       <c r="O59" s="4"/>
     </row>
-    <row r="60" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B60" s="14"/>
-      <c r="J60" s="14"/>
-      <c r="K60" s="14"/>
-      <c r="L60" s="13"/>
+    <row r="60" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L60" s="4"/>
       <c r="M60" s="4"/>
       <c r="N60" s="4"/>
       <c r="O60" s="4"/>
     </row>
-    <row r="61" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B61" s="14"/>
-      <c r="J61" s="14"/>
-      <c r="K61" s="14"/>
-      <c r="L61" s="13"/>
+    <row r="61" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L61" s="4"/>
       <c r="M61" s="4"/>
       <c r="N61" s="4"/>
       <c r="O61" s="4"/>
     </row>
-    <row r="62" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B62" s="14"/>
-      <c r="J62" s="14"/>
-      <c r="K62" s="14"/>
-      <c r="L62" s="13"/>
+    <row r="62" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L62" s="4"/>
       <c r="M62" s="4"/>
       <c r="N62" s="4"/>
       <c r="O62" s="4"/>
     </row>
-    <row r="63" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B63" s="14"/>
-      <c r="J63" s="14"/>
-      <c r="K63" s="14"/>
-      <c r="L63" s="13"/>
+    <row r="63" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L63" s="4"/>
       <c r="M63" s="4"/>
       <c r="N63" s="4"/>
       <c r="O63" s="4"/>
     </row>
-    <row r="64" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B64" s="14"/>
-      <c r="J64" s="14"/>
-      <c r="K64" s="14"/>
-      <c r="L64" s="13"/>
+    <row r="64" spans="12:15" x14ac:dyDescent="0.3">
+      <c r="L64" s="4"/>
       <c r="M64" s="4"/>
       <c r="N64" s="4"/>
       <c r="O64" s="4"/>
     </row>
-    <row r="65" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B65" s="14"/>
-      <c r="J65" s="14"/>
-      <c r="K65" s="14"/>
-      <c r="L65" s="13"/>
+    <row r="65" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="L65" s="4"/>
       <c r="M65" s="4"/>
       <c r="N65" s="4"/>
       <c r="O65" s="4"/>
     </row>
-    <row r="66" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B66" s="14"/>
-      <c r="J66" s="14"/>
-      <c r="K66" s="14"/>
-      <c r="L66" s="13"/>
+    <row r="66" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="L66" s="4"/>
       <c r="M66" s="4"/>
       <c r="N66" s="4"/>
       <c r="O66" s="4"/>
     </row>
-    <row r="67" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B67" s="14"/>
-      <c r="J67" s="14"/>
-      <c r="K67" s="14"/>
-      <c r="L67" s="13"/>
+    <row r="67" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="L67" s="4"/>
       <c r="M67" s="4"/>
       <c r="N67" s="4"/>
       <c r="O67" s="4"/>
     </row>
-    <row r="68" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B68" s="14"/>
-      <c r="J68" s="14"/>
-      <c r="K68" s="14"/>
-      <c r="L68" s="13"/>
+    <row r="68" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="L68" s="4"/>
       <c r="M68" s="4"/>
       <c r="N68" s="4"/>
       <c r="O68" s="4"/>
     </row>
-    <row r="69" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B69" s="14"/>
-      <c r="J69" s="14"/>
-      <c r="K69" s="14"/>
-      <c r="L69" s="13"/>
+    <row r="69" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="L69" s="4"/>
       <c r="M69" s="4"/>
       <c r="N69" s="4"/>
       <c r="O69" s="4"/>
     </row>
-    <row r="70" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B70" s="14"/>
-      <c r="J70" s="14"/>
-      <c r="K70" s="14"/>
-      <c r="L70" s="13"/>
+    <row r="70" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="L70" s="4"/>
       <c r="M70" s="4"/>
       <c r="N70" s="4"/>
       <c r="O70" s="4"/>
     </row>
-    <row r="71" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B71" s="14"/>
-      <c r="J71" s="14"/>
-      <c r="K71" s="14"/>
-      <c r="L71" s="13"/>
+    <row r="71" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="L71" s="4"/>
       <c r="M71" s="4"/>
       <c r="N71" s="4"/>
       <c r="O71" s="4"/>
     </row>
-    <row r="72" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B72" s="14"/>
-      <c r="J72" s="14"/>
-      <c r="K72" s="14"/>
-      <c r="L72" s="13"/>
+    <row r="72" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="L72" s="4"/>
       <c r="M72" s="4"/>
       <c r="N72" s="4"/>
       <c r="O72" s="4"/>
     </row>
-    <row r="73" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B73" s="14"/>
-      <c r="J73" s="14"/>
-      <c r="K73" s="14"/>
-      <c r="L73" s="13"/>
+    <row r="73" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="L73" s="4"/>
       <c r="M73" s="4"/>
       <c r="N73" s="4"/>
       <c r="O73" s="4"/>
     </row>
-    <row r="74" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B74" s="14"/>
-      <c r="J74" s="14"/>
-      <c r="K74" s="14"/>
-      <c r="L74" s="13"/>
+    <row r="74" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="L74" s="4"/>
       <c r="M74" s="4"/>
       <c r="N74" s="4"/>
       <c r="O74" s="4"/>
     </row>
-    <row r="75" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B75" s="14"/>
-      <c r="J75" s="14"/>
-      <c r="K75" s="14"/>
-      <c r="L75" s="13"/>
+    <row r="75" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="L75" s="4"/>
       <c r="M75" s="4"/>
       <c r="N75" s="4"/>
       <c r="O75" s="4"/>
     </row>
-    <row r="76" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B76" s="14"/>
-      <c r="J76" s="14"/>
-      <c r="K76" s="14"/>
-      <c r="L76" s="13"/>
+    <row r="76" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="L76" s="4"/>
       <c r="M76" s="4"/>
       <c r="N76" s="4"/>
       <c r="O76" s="4"/>
     </row>
-    <row r="77" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B77" s="14"/>
-      <c r="J77" s="14"/>
-      <c r="K77" s="14"/>
-      <c r="L77" s="12"/>
-    </row>
-    <row r="78" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B78" s="14"/>
+    <row r="78" spans="8:15" x14ac:dyDescent="0.3">
       <c r="H78" s="4"/>
       <c r="I78" s="4"/>
-      <c r="J78" s="13"/>
-      <c r="K78" s="14"/>
-    </row>
-    <row r="79" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B79" s="14"/>
-      <c r="J79" s="14"/>
-      <c r="K79" s="14"/>
-    </row>
-    <row r="80" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B80" s="14"/>
-      <c r="J80" s="14"/>
-      <c r="K80" s="14"/>
-    </row>
-    <row r="81" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B81" s="14"/>
-      <c r="J81" s="14"/>
-      <c r="K81" s="14"/>
-    </row>
-    <row r="82" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B82" s="14"/>
-      <c r="J82" s="14"/>
-      <c r="K82" s="14"/>
-    </row>
-    <row r="83" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B83" s="14"/>
-      <c r="J83" s="14"/>
-      <c r="K83" s="14"/>
-    </row>
-    <row r="84" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B84" s="14"/>
-      <c r="J84" s="14"/>
-      <c r="K84" s="14"/>
-    </row>
-    <row r="85" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B85" s="14"/>
-      <c r="J85" s="14"/>
-      <c r="K85" s="14"/>
-    </row>
-    <row r="86" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B86" s="14"/>
-      <c r="J86" s="14"/>
-      <c r="K86" s="14"/>
-    </row>
-    <row r="87" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B87" s="14"/>
-      <c r="J87" s="14"/>
-      <c r="K87" s="14"/>
-    </row>
-    <row r="88" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B88" s="14"/>
-      <c r="J88" s="14"/>
-      <c r="K88" s="14"/>
-    </row>
-    <row r="89" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B89" s="14"/>
-      <c r="J89" s="14"/>
-      <c r="K89" s="14"/>
-    </row>
-    <row r="90" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B90" s="14"/>
-      <c r="J90" s="14"/>
-      <c r="K90" s="14"/>
-    </row>
-    <row r="91" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B91" s="14"/>
-      <c r="J91" s="14"/>
-      <c r="K91" s="14"/>
-    </row>
-    <row r="92" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B92" s="14"/>
-      <c r="J92" s="14"/>
-      <c r="K92" s="14"/>
-    </row>
-    <row r="93" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B93" s="14"/>
-      <c r="J93" s="14"/>
-      <c r="K93" s="14"/>
-    </row>
-    <row r="94" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B94" s="14"/>
-      <c r="J94" s="14"/>
-      <c r="K94" s="14"/>
-    </row>
-    <row r="95" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B95" s="14"/>
-      <c r="J95" s="14"/>
-      <c r="K95" s="14"/>
-    </row>
-    <row r="96" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B96" s="14"/>
-      <c r="J96" s="14"/>
-      <c r="K96" s="14"/>
-    </row>
-    <row r="97" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B97" s="14"/>
-      <c r="J97" s="14"/>
-      <c r="K97" s="14"/>
-    </row>
-    <row r="98" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B98" s="14"/>
-      <c r="J98" s="14"/>
-      <c r="K98" s="14"/>
-    </row>
-    <row r="99" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B99" s="14"/>
-      <c r="J99" s="14"/>
-      <c r="K99" s="14"/>
-    </row>
-    <row r="100" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B100" s="14"/>
-      <c r="J100" s="14"/>
-      <c r="K100" s="14"/>
-    </row>
-    <row r="101" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B101" s="14"/>
-      <c r="J101" s="14"/>
-      <c r="K101" s="14"/>
-    </row>
-    <row r="102" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B102" s="14"/>
-      <c r="J102" s="14"/>
-      <c r="K102" s="14"/>
-    </row>
-    <row r="103" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B103" s="14"/>
-    </row>
-    <row r="104" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B104" s="14"/>
-    </row>
-    <row r="105" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B105" s="14"/>
-    </row>
-    <row r="106" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B106" s="14"/>
-    </row>
-    <row r="107" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B107" s="14"/>
-    </row>
-    <row r="108" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B108" s="14"/>
-    </row>
-    <row r="109" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B109" s="14"/>
-    </row>
-    <row r="110" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B110" s="14"/>
-    </row>
-    <row r="111" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B111" s="14"/>
-    </row>
-    <row r="112" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B112" s="14"/>
-    </row>
-    <row r="113" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B113" s="14"/>
-    </row>
-    <row r="114" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B114" s="14"/>
-    </row>
-    <row r="115" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B115" s="14"/>
-    </row>
-    <row r="116" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B116" s="14"/>
-    </row>
-    <row r="117" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B117" s="14"/>
-    </row>
-    <row r="118" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B118" s="14"/>
-    </row>
-    <row r="119" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B119" s="14"/>
-    </row>
-    <row r="120" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B120" s="14"/>
-    </row>
-    <row r="121" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B121" s="14"/>
-    </row>
-    <row r="122" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B122" s="14"/>
-    </row>
-    <row r="123" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B123" s="14"/>
-    </row>
-    <row r="124" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B124" s="14"/>
-    </row>
-    <row r="125" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B125" s="14"/>
-    </row>
-    <row r="126" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B126" s="14"/>
-    </row>
-    <row r="127" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B127" s="14"/>
-    </row>
-    <row r="128" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B128" s="14"/>
-    </row>
-    <row r="129" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B129" s="14"/>
-    </row>
-    <row r="130" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B130" s="14"/>
-    </row>
-    <row r="131" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B131" s="14"/>
-    </row>
-    <row r="132" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B132" s="14"/>
-    </row>
-    <row r="133" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B133" s="14"/>
-    </row>
-    <row r="134" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B134" s="14"/>
-    </row>
-    <row r="135" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B135" s="14"/>
-    </row>
-    <row r="136" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B136" s="14"/>
-    </row>
-    <row r="137" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B137" s="14"/>
-    </row>
-    <row r="138" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B138" s="14"/>
-    </row>
-    <row r="139" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B139" s="14"/>
-    </row>
-    <row r="140" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B140" s="14"/>
-    </row>
-    <row r="141" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B141" s="14"/>
-    </row>
-    <row r="142" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B142" s="14"/>
-    </row>
-    <row r="143" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B143" s="14"/>
+      <c r="J78" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="57" fitToHeight="72" orientation="portrait" r:id="rId1"/>
   <headerFooter>
-    <oddHeader>&amp;A</oddHeader>
+    <oddHeader>&amp;LUBA Test Report&amp;R&amp;D</oddHeader>
     <oddFooter>Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <rowBreaks count="2" manualBreakCount="2">

</xml_diff>

<commit_message>
bug 29,32: PDF file full name, font, test indices start from 1
</commit_message>
<xml_diff>
--- a/web-console/server/assets/pdf_template.xlsx
+++ b/web-console/server/assets/pdf_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\DEV\UBA6\web-console\server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FDEBAEB-E12F-4A4F-92EF-492B61E60570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C22BBFF-CC12-4544-82E9-81B0F532ECE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
   <si>
     <t>Wh</t>
   </si>
@@ -136,12 +136,15 @@
   <si>
     <t>Parallel</t>
   </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -189,7 +192,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
+      <b/>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="13"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -218,13 +229,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -239,8 +247,12 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5652,8 +5664,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="605922" y="380713"/>
-          <a:ext cx="9312753" cy="4137009"/>
+          <a:off x="612272" y="387063"/>
+          <a:ext cx="9595328" cy="4314809"/>
           <a:chOff x="614350" y="401783"/>
           <a:chExt cx="9325165" cy="4265799"/>
         </a:xfrm>
@@ -6121,10 +6133,12 @@
     <col min="1" max="1" width="7.44140625" style="2" customWidth="1"/>
     <col min="2" max="2" width="2.109375" style="2" customWidth="1"/>
     <col min="3" max="3" width="2.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="9" width="19.6640625" style="2" customWidth="1"/>
+    <col min="4" max="7" width="19.6640625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="23.6640625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="19.6640625" style="2" customWidth="1"/>
     <col min="10" max="10" width="9.44140625" style="2" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="4.109375" style="2" customWidth="1"/>
-    <col min="12" max="12" width="9.109375" style="8"/>
+    <col min="12" max="12" width="9.109375" style="7"/>
     <col min="13" max="13" width="82.44140625" style="2" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="123.33203125" style="2" customWidth="1"/>
     <col min="15" max="15" width="78.88671875" style="2" customWidth="1"/>
@@ -6132,646 +6146,826 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:14" ht="8.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="J2" s="4"/>
-    </row>
-    <row r="3" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B3" s="4"/>
-      <c r="D3" s="3" t="s">
+      <c r="J2" s="3"/>
+    </row>
+    <row r="3" spans="2:14" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="B3" s="3"/>
+      <c r="D3" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="3" t="s">
+      <c r="E3" s="10"/>
+      <c r="F3" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="G3" s="11"/>
+      <c r="H3" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="I3" s="11"/>
+      <c r="J3" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="K3" s="4"/>
-      <c r="N3" s="5"/>
+      <c r="K3" s="3"/>
+      <c r="N3" s="4"/>
     </row>
     <row r="4" spans="2:14" ht="5.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="4"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="N4" s="5"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="N4" s="4"/>
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="9"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="8"/>
+      <c r="I5" s="8"/>
+      <c r="J5" s="8"/>
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="9"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="9"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="9"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="9"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
     </row>
     <row r="18" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="9"/>
-      <c r="H18" s="9"/>
-      <c r="I18" s="9"/>
-      <c r="J18" s="9"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8"/>
     </row>
     <row r="19" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="9"/>
-      <c r="J19" s="9"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="8"/>
     </row>
     <row r="20" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="9"/>
-      <c r="J20" s="9"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="8"/>
+      <c r="J20" s="8"/>
     </row>
     <row r="21" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="9"/>
-      <c r="H21" s="9"/>
-      <c r="I21" s="9"/>
-      <c r="J21" s="9"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="8"/>
+      <c r="J21" s="8"/>
     </row>
     <row r="22" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
-      <c r="G22" s="9"/>
-      <c r="H22" s="9"/>
-      <c r="I22" s="9"/>
-      <c r="J22" s="9"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8"/>
+      <c r="I22" s="8"/>
+      <c r="J22" s="8"/>
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="9"/>
-      <c r="H23" s="9"/>
-      <c r="I23" s="9"/>
-      <c r="J23" s="9"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
+      <c r="J23" s="8"/>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
-      <c r="I24" s="9"/>
-      <c r="J24" s="9"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="8"/>
+      <c r="H24" s="8"/>
+      <c r="I24" s="8"/>
+      <c r="J24" s="8"/>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="9"/>
-      <c r="H25" s="9"/>
-      <c r="I25" s="9"/>
-      <c r="J25" s="9"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="8"/>
+      <c r="I25" s="8"/>
+      <c r="J25" s="8"/>
     </row>
     <row r="26" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="9"/>
-      <c r="H26" s="9"/>
-      <c r="I26" s="9"/>
-      <c r="J26" s="9"/>
-      <c r="M26" s="7"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="8"/>
+      <c r="I26" s="8"/>
+      <c r="J26" s="8"/>
+      <c r="M26" s="6"/>
     </row>
     <row r="28" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B28" s="4"/>
-      <c r="K28" s="4"/>
-    </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="D29" s="4" t="s">
+      <c r="B28" s="3"/>
+      <c r="K28" s="3"/>
+    </row>
+    <row r="29" spans="2:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D29" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
-      <c r="G29" s="4"/>
-      <c r="H29" s="4" t="s">
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="I29" s="4"/>
-      <c r="J29" s="4"/>
-    </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="D30" s="2" t="s">
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+    </row>
+    <row r="30" spans="2:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D30" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="H30" s="2" t="s">
+      <c r="E30" s="11"/>
+      <c r="F30" s="11"/>
+      <c r="G30" s="11"/>
+      <c r="H30" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I30" s="10"/>
-      <c r="L30" s="4"/>
-      <c r="M30" s="4"/>
-      <c r="N30" s="4"/>
-      <c r="O30" s="4"/>
-    </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="H31" s="2" t="s">
+      <c r="I30" s="11"/>
+      <c r="J30" s="11"/>
+      <c r="L30" s="3"/>
+      <c r="M30" s="3"/>
+      <c r="N30" s="3"/>
+      <c r="O30" s="3"/>
+    </row>
+    <row r="31" spans="2:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D31" s="11"/>
+      <c r="E31" s="11"/>
+      <c r="F31" s="11"/>
+      <c r="G31" s="11"/>
+      <c r="H31" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="I31" s="10"/>
-      <c r="L31" s="4"/>
-      <c r="M31" s="4"/>
-      <c r="N31" s="4"/>
-      <c r="O31" s="4"/>
-    </row>
-    <row r="32" spans="2:15" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="D32" s="2" t="s">
+      <c r="I31" s="11"/>
+      <c r="J31" s="11"/>
+      <c r="L31" s="3"/>
+      <c r="M31" s="3"/>
+      <c r="N31" s="3"/>
+      <c r="O31" s="3"/>
+    </row>
+    <row r="32" spans="2:15" s="3" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D32" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
-      <c r="G32" s="2"/>
-      <c r="H32" s="2" t="s">
+      <c r="E32" s="11"/>
+      <c r="F32" s="11"/>
+      <c r="G32" s="11"/>
+      <c r="H32" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="I32" s="10"/>
-      <c r="J32" s="2"/>
-    </row>
-    <row r="33" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="D33" s="2" t="s">
+      <c r="I32" s="11"/>
+      <c r="J32" s="11"/>
+    </row>
+    <row r="33" spans="3:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D33" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="H33" s="2" t="s">
+      <c r="E33" s="11"/>
+      <c r="F33" s="11"/>
+      <c r="G33" s="11"/>
+      <c r="H33" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="I33" s="10"/>
-      <c r="J33" s="2" t="s">
+      <c r="I33" s="11"/>
+      <c r="J33" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="L33" s="4"/>
-      <c r="M33" s="4"/>
-      <c r="N33" s="4"/>
-      <c r="O33" s="4"/>
-    </row>
-    <row r="34" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="H34" s="2" t="s">
+      <c r="L33" s="3"/>
+      <c r="M33" s="3"/>
+      <c r="N33" s="3"/>
+      <c r="O33" s="3"/>
+    </row>
+    <row r="34" spans="3:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D34" s="11"/>
+      <c r="E34" s="11"/>
+      <c r="F34" s="11"/>
+      <c r="G34" s="11"/>
+      <c r="H34" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="I34" s="10"/>
-      <c r="J34" s="2" t="s">
+      <c r="I34" s="11"/>
+      <c r="J34" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="L34" s="4"/>
-      <c r="M34" s="4"/>
-      <c r="N34" s="4"/>
-      <c r="O34" s="4"/>
-    </row>
-    <row r="35" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="H35" s="2" t="s">
+      <c r="L34" s="3"/>
+      <c r="M34" s="3"/>
+      <c r="N34" s="3"/>
+      <c r="O34" s="3"/>
+    </row>
+    <row r="35" spans="3:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D35" s="11"/>
+      <c r="E35" s="11"/>
+      <c r="F35" s="11"/>
+      <c r="G35" s="11"/>
+      <c r="H35" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="I35" s="10"/>
-      <c r="J35" s="2" t="s">
+      <c r="I35" s="11"/>
+      <c r="J35" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="L35" s="4"/>
-      <c r="M35" s="4"/>
-      <c r="N35" s="4"/>
-      <c r="O35" s="4"/>
-    </row>
-    <row r="36" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="H36" s="2" t="s">
+      <c r="L35" s="3"/>
+      <c r="M35" s="3"/>
+      <c r="N35" s="3"/>
+      <c r="O35" s="3"/>
+    </row>
+    <row r="36" spans="3:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D36" s="11"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="11"/>
+      <c r="G36" s="11"/>
+      <c r="H36" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="I36" s="10"/>
-      <c r="L36" s="4"/>
-      <c r="M36" s="4"/>
-      <c r="N36" s="4"/>
-      <c r="O36" s="4"/>
-    </row>
-    <row r="37" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="D37" s="2" t="s">
+      <c r="I36" s="11"/>
+      <c r="J36" s="11"/>
+      <c r="L36" s="3"/>
+      <c r="M36" s="3"/>
+      <c r="N36" s="3"/>
+      <c r="O36" s="3"/>
+    </row>
+    <row r="37" spans="3:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D37" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="H37" s="2" t="s">
+      <c r="E37" s="11"/>
+      <c r="F37" s="11"/>
+      <c r="G37" s="11"/>
+      <c r="H37" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="I37" s="10"/>
-      <c r="L37" s="4"/>
-      <c r="M37" s="4"/>
-      <c r="N37" s="4"/>
-      <c r="O37" s="4"/>
-    </row>
-    <row r="38" spans="3:15" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="D38" s="2" t="s">
+      <c r="I37" s="11"/>
+      <c r="J37" s="11"/>
+      <c r="L37" s="3"/>
+      <c r="M37" s="3"/>
+      <c r="N37" s="3"/>
+      <c r="O37" s="3"/>
+    </row>
+    <row r="38" spans="3:15" s="3" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D38" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="E38" s="2"/>
-      <c r="F38" s="2"/>
-      <c r="G38" s="2"/>
-      <c r="H38" s="2" t="s">
+      <c r="E38" s="11"/>
+      <c r="F38" s="11"/>
+      <c r="G38" s="11"/>
+      <c r="H38" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="I38" s="10"/>
-      <c r="J38" s="2"/>
-    </row>
-    <row r="39" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="D39" s="4" t="s">
+      <c r="I38" s="11"/>
+      <c r="J38" s="11"/>
+    </row>
+    <row r="39" spans="3:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D39" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E39" s="4"/>
-      <c r="F39" s="4"/>
-      <c r="G39" s="4"/>
-      <c r="H39" s="4"/>
-      <c r="I39" s="4"/>
-      <c r="J39" s="4"/>
-      <c r="L39" s="4"/>
-      <c r="M39" s="4"/>
-      <c r="N39" s="4"/>
-      <c r="O39" s="4"/>
-    </row>
-    <row r="40" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="L40" s="4"/>
-      <c r="M40" s="4"/>
-      <c r="N40" s="4"/>
-      <c r="O40" s="4"/>
-    </row>
-    <row r="41" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="C41" s="2">
-        <v>1</v>
+      <c r="E39" s="10"/>
+      <c r="F39" s="10"/>
+      <c r="G39" s="10"/>
+      <c r="H39" s="10"/>
+      <c r="I39" s="10"/>
+      <c r="J39" s="10"/>
+      <c r="L39" s="3"/>
+      <c r="M39" s="3"/>
+      <c r="N39" s="3"/>
+      <c r="O39" s="3"/>
+    </row>
+    <row r="40" spans="3:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D40" s="11"/>
+      <c r="E40" s="11"/>
+      <c r="F40" s="11"/>
+      <c r="G40" s="11"/>
+      <c r="H40" s="11"/>
+      <c r="I40" s="11"/>
+      <c r="J40" s="11"/>
+      <c r="L40" s="3"/>
+      <c r="M40" s="3"/>
+      <c r="N40" s="3"/>
+      <c r="O40" s="3"/>
+    </row>
+    <row r="41" spans="3:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="C41" s="2" t="s">
+        <v>31</v>
       </c>
-      <c r="D41" s="4"/>
-      <c r="G41" s="4"/>
-      <c r="H41" s="4" t="s">
+      <c r="D41" s="10"/>
+      <c r="E41" s="11"/>
+      <c r="F41" s="11"/>
+      <c r="G41" s="10"/>
+      <c r="H41" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="I41" s="4"/>
-      <c r="J41" s="4"/>
-      <c r="L41" s="4"/>
-      <c r="M41" s="4"/>
-      <c r="N41" s="4"/>
-      <c r="O41" s="4"/>
-    </row>
-    <row r="42" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="L42" s="4"/>
-      <c r="M42" s="4"/>
-      <c r="N42" s="4"/>
-      <c r="O42" s="4"/>
-    </row>
-    <row r="43" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="L43" s="4"/>
-      <c r="M43" s="4"/>
-      <c r="N43" s="4"/>
-      <c r="O43" s="4"/>
-    </row>
-    <row r="44" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="L44" s="4"/>
-      <c r="M44" s="4"/>
-      <c r="N44" s="4"/>
-      <c r="O44" s="4"/>
-    </row>
-    <row r="45" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="L45" s="4"/>
-      <c r="M45" s="4"/>
-      <c r="N45" s="4"/>
-      <c r="O45" s="4"/>
-    </row>
-    <row r="46" spans="3:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="L46" s="4"/>
-      <c r="M46" s="4"/>
-      <c r="N46" s="4"/>
-      <c r="O46" s="4"/>
-    </row>
-    <row r="47" spans="3:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="L47" s="4"/>
-      <c r="M47" s="4"/>
-      <c r="N47" s="4"/>
-      <c r="O47" s="4"/>
-    </row>
-    <row r="48" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="L48" s="4"/>
-      <c r="M48" s="4"/>
-      <c r="N48" s="4"/>
-      <c r="O48" s="4"/>
-    </row>
-    <row r="49" spans="12:15" x14ac:dyDescent="0.3">
-      <c r="L49" s="4"/>
-      <c r="M49" s="4"/>
-      <c r="N49" s="4"/>
-      <c r="O49" s="4"/>
-    </row>
-    <row r="50" spans="12:15" x14ac:dyDescent="0.3">
-      <c r="L50" s="4"/>
-      <c r="M50" s="4"/>
-      <c r="N50" s="4"/>
-      <c r="O50" s="4"/>
-    </row>
-    <row r="51" spans="12:15" x14ac:dyDescent="0.3">
-      <c r="L51" s="4"/>
-      <c r="M51" s="4"/>
-      <c r="N51" s="4"/>
-      <c r="O51" s="4"/>
-    </row>
-    <row r="52" spans="12:15" x14ac:dyDescent="0.3">
-      <c r="L52" s="4"/>
-      <c r="M52" s="4"/>
-      <c r="N52" s="4"/>
-      <c r="O52" s="4"/>
-    </row>
-    <row r="53" spans="12:15" x14ac:dyDescent="0.3">
-      <c r="L53" s="4"/>
-      <c r="M53" s="4"/>
-      <c r="N53" s="4"/>
-      <c r="O53" s="4"/>
-    </row>
-    <row r="54" spans="12:15" x14ac:dyDescent="0.3">
-      <c r="L54" s="4"/>
-      <c r="M54" s="4"/>
-      <c r="N54" s="4"/>
-      <c r="O54" s="4"/>
-    </row>
-    <row r="55" spans="12:15" x14ac:dyDescent="0.3">
-      <c r="L55" s="4"/>
-      <c r="M55" s="4"/>
-      <c r="N55" s="4"/>
-      <c r="O55" s="4"/>
-    </row>
-    <row r="56" spans="12:15" x14ac:dyDescent="0.3">
-      <c r="L56" s="4"/>
-      <c r="M56" s="4"/>
-      <c r="N56" s="4"/>
-      <c r="O56" s="4"/>
-    </row>
-    <row r="57" spans="12:15" x14ac:dyDescent="0.3">
-      <c r="L57" s="4"/>
-      <c r="M57" s="4"/>
-      <c r="N57" s="4"/>
-      <c r="O57" s="4"/>
-    </row>
-    <row r="58" spans="12:15" x14ac:dyDescent="0.3">
-      <c r="L58" s="4"/>
-      <c r="M58" s="4"/>
-      <c r="N58" s="4"/>
-      <c r="O58" s="4"/>
-    </row>
-    <row r="59" spans="12:15" x14ac:dyDescent="0.3">
-      <c r="L59" s="4"/>
-      <c r="M59" s="4"/>
-      <c r="N59" s="4"/>
-      <c r="O59" s="4"/>
-    </row>
-    <row r="60" spans="12:15" x14ac:dyDescent="0.3">
-      <c r="L60" s="4"/>
-      <c r="M60" s="4"/>
-      <c r="N60" s="4"/>
-      <c r="O60" s="4"/>
-    </row>
-    <row r="61" spans="12:15" x14ac:dyDescent="0.3">
-      <c r="L61" s="4"/>
-      <c r="M61" s="4"/>
-      <c r="N61" s="4"/>
-      <c r="O61" s="4"/>
-    </row>
-    <row r="62" spans="12:15" x14ac:dyDescent="0.3">
-      <c r="L62" s="4"/>
-      <c r="M62" s="4"/>
-      <c r="N62" s="4"/>
-      <c r="O62" s="4"/>
-    </row>
-    <row r="63" spans="12:15" x14ac:dyDescent="0.3">
-      <c r="L63" s="4"/>
-      <c r="M63" s="4"/>
-      <c r="N63" s="4"/>
-      <c r="O63" s="4"/>
-    </row>
-    <row r="64" spans="12:15" x14ac:dyDescent="0.3">
-      <c r="L64" s="4"/>
-      <c r="M64" s="4"/>
-      <c r="N64" s="4"/>
-      <c r="O64" s="4"/>
+      <c r="I41" s="10"/>
+      <c r="J41" s="10"/>
+      <c r="L41" s="3"/>
+      <c r="M41" s="3"/>
+      <c r="N41" s="3"/>
+      <c r="O41" s="3"/>
+    </row>
+    <row r="42" spans="3:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D42" s="11"/>
+      <c r="E42" s="11"/>
+      <c r="F42" s="11"/>
+      <c r="G42" s="11"/>
+      <c r="H42" s="11"/>
+      <c r="I42" s="11"/>
+      <c r="J42" s="11"/>
+      <c r="L42" s="3"/>
+      <c r="M42" s="3"/>
+      <c r="N42" s="3"/>
+      <c r="O42" s="3"/>
+    </row>
+    <row r="43" spans="3:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D43" s="11"/>
+      <c r="E43" s="11"/>
+      <c r="F43" s="11"/>
+      <c r="G43" s="11"/>
+      <c r="H43" s="11"/>
+      <c r="I43" s="11"/>
+      <c r="J43" s="11"/>
+      <c r="L43" s="3"/>
+      <c r="M43" s="3"/>
+      <c r="N43" s="3"/>
+      <c r="O43" s="3"/>
+    </row>
+    <row r="44" spans="3:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D44" s="11"/>
+      <c r="E44" s="11"/>
+      <c r="F44" s="11"/>
+      <c r="G44" s="11"/>
+      <c r="H44" s="11"/>
+      <c r="I44" s="11"/>
+      <c r="J44" s="11"/>
+      <c r="L44" s="3"/>
+      <c r="M44" s="3"/>
+      <c r="N44" s="3"/>
+      <c r="O44" s="3"/>
+    </row>
+    <row r="45" spans="3:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D45" s="11"/>
+      <c r="E45" s="11"/>
+      <c r="F45" s="11"/>
+      <c r="G45" s="11"/>
+      <c r="H45" s="11"/>
+      <c r="I45" s="11"/>
+      <c r="J45" s="11"/>
+      <c r="L45" s="3"/>
+      <c r="M45" s="3"/>
+      <c r="N45" s="3"/>
+      <c r="O45" s="3"/>
+    </row>
+    <row r="46" spans="3:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D46" s="11"/>
+      <c r="E46" s="11"/>
+      <c r="F46" s="11"/>
+      <c r="G46" s="11"/>
+      <c r="H46" s="11"/>
+      <c r="I46" s="11"/>
+      <c r="J46" s="11"/>
+      <c r="L46" s="3"/>
+      <c r="M46" s="3"/>
+      <c r="N46" s="3"/>
+      <c r="O46" s="3"/>
+    </row>
+    <row r="47" spans="3:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D47" s="11"/>
+      <c r="E47" s="11"/>
+      <c r="F47" s="11"/>
+      <c r="G47" s="11"/>
+      <c r="H47" s="11"/>
+      <c r="I47" s="11"/>
+      <c r="J47" s="11"/>
+      <c r="L47" s="3"/>
+      <c r="M47" s="3"/>
+      <c r="N47" s="3"/>
+      <c r="O47" s="3"/>
+    </row>
+    <row r="48" spans="3:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D48" s="11"/>
+      <c r="E48" s="11"/>
+      <c r="F48" s="11"/>
+      <c r="G48" s="11"/>
+      <c r="H48" s="11"/>
+      <c r="I48" s="11"/>
+      <c r="J48" s="11"/>
+      <c r="L48" s="3"/>
+      <c r="M48" s="3"/>
+      <c r="N48" s="3"/>
+      <c r="O48" s="3"/>
+    </row>
+    <row r="49" spans="4:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D49" s="11"/>
+      <c r="E49" s="11"/>
+      <c r="F49" s="11"/>
+      <c r="G49" s="11"/>
+      <c r="H49" s="11"/>
+      <c r="I49" s="11"/>
+      <c r="J49" s="11"/>
+      <c r="L49" s="3"/>
+      <c r="M49" s="3"/>
+      <c r="N49" s="3"/>
+      <c r="O49" s="3"/>
+    </row>
+    <row r="50" spans="4:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D50" s="11"/>
+      <c r="E50" s="11"/>
+      <c r="F50" s="11"/>
+      <c r="G50" s="11"/>
+      <c r="H50" s="11"/>
+      <c r="I50" s="11"/>
+      <c r="J50" s="11"/>
+      <c r="L50" s="3"/>
+      <c r="M50" s="3"/>
+      <c r="N50" s="3"/>
+      <c r="O50" s="3"/>
+    </row>
+    <row r="51" spans="4:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D51" s="11"/>
+      <c r="E51" s="11"/>
+      <c r="F51" s="11"/>
+      <c r="G51" s="11"/>
+      <c r="H51" s="11"/>
+      <c r="I51" s="11"/>
+      <c r="J51" s="11"/>
+      <c r="L51" s="3"/>
+      <c r="M51" s="3"/>
+      <c r="N51" s="3"/>
+      <c r="O51" s="3"/>
+    </row>
+    <row r="52" spans="4:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D52" s="11"/>
+      <c r="E52" s="11"/>
+      <c r="F52" s="11"/>
+      <c r="G52" s="11"/>
+      <c r="H52" s="11"/>
+      <c r="I52" s="11"/>
+      <c r="J52" s="11"/>
+      <c r="L52" s="3"/>
+      <c r="M52" s="3"/>
+      <c r="N52" s="3"/>
+      <c r="O52" s="3"/>
+    </row>
+    <row r="53" spans="4:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D53" s="11"/>
+      <c r="E53" s="11"/>
+      <c r="F53" s="11"/>
+      <c r="G53" s="11"/>
+      <c r="H53" s="11"/>
+      <c r="I53" s="11"/>
+      <c r="J53" s="11"/>
+      <c r="L53" s="3"/>
+      <c r="M53" s="3"/>
+      <c r="N53" s="3"/>
+      <c r="O53" s="3"/>
+    </row>
+    <row r="54" spans="4:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D54" s="11"/>
+      <c r="E54" s="11"/>
+      <c r="F54" s="11"/>
+      <c r="G54" s="11"/>
+      <c r="H54" s="11"/>
+      <c r="I54" s="11"/>
+      <c r="J54" s="11"/>
+      <c r="L54" s="3"/>
+      <c r="M54" s="3"/>
+      <c r="N54" s="3"/>
+      <c r="O54" s="3"/>
+    </row>
+    <row r="55" spans="4:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D55" s="11"/>
+      <c r="E55" s="11"/>
+      <c r="F55" s="11"/>
+      <c r="G55" s="11"/>
+      <c r="H55" s="11"/>
+      <c r="I55" s="11"/>
+      <c r="J55" s="11"/>
+      <c r="L55" s="3"/>
+      <c r="M55" s="3"/>
+      <c r="N55" s="3"/>
+      <c r="O55" s="3"/>
+    </row>
+    <row r="56" spans="4:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D56" s="11"/>
+      <c r="E56" s="11"/>
+      <c r="F56" s="11"/>
+      <c r="G56" s="11"/>
+      <c r="H56" s="11"/>
+      <c r="I56" s="11"/>
+      <c r="J56" s="11"/>
+      <c r="L56" s="3"/>
+      <c r="M56" s="3"/>
+      <c r="N56" s="3"/>
+      <c r="O56" s="3"/>
+    </row>
+    <row r="57" spans="4:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D57" s="11"/>
+      <c r="E57" s="11"/>
+      <c r="F57" s="11"/>
+      <c r="G57" s="11"/>
+      <c r="H57" s="11"/>
+      <c r="I57" s="11"/>
+      <c r="J57" s="11"/>
+      <c r="L57" s="3"/>
+      <c r="M57" s="3"/>
+      <c r="N57" s="3"/>
+      <c r="O57" s="3"/>
+    </row>
+    <row r="58" spans="4:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D58" s="11"/>
+      <c r="E58" s="11"/>
+      <c r="F58" s="11"/>
+      <c r="G58" s="11"/>
+      <c r="H58" s="11"/>
+      <c r="I58" s="11"/>
+      <c r="J58" s="11"/>
+      <c r="L58" s="3"/>
+      <c r="M58" s="3"/>
+      <c r="N58" s="3"/>
+      <c r="O58" s="3"/>
+    </row>
+    <row r="59" spans="4:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D59" s="11"/>
+      <c r="E59" s="11"/>
+      <c r="F59" s="11"/>
+      <c r="G59" s="11"/>
+      <c r="H59" s="11"/>
+      <c r="I59" s="11"/>
+      <c r="J59" s="11"/>
+      <c r="L59" s="3"/>
+      <c r="M59" s="3"/>
+      <c r="N59" s="3"/>
+      <c r="O59" s="3"/>
+    </row>
+    <row r="60" spans="4:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D60" s="11"/>
+      <c r="E60" s="11"/>
+      <c r="F60" s="11"/>
+      <c r="G60" s="11"/>
+      <c r="H60" s="11"/>
+      <c r="I60" s="11"/>
+      <c r="J60" s="11"/>
+      <c r="L60" s="3"/>
+      <c r="M60" s="3"/>
+      <c r="N60" s="3"/>
+      <c r="O60" s="3"/>
+    </row>
+    <row r="61" spans="4:15" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="D61" s="11"/>
+      <c r="E61" s="11"/>
+      <c r="F61" s="11"/>
+      <c r="G61" s="11"/>
+      <c r="H61" s="11"/>
+      <c r="I61" s="11"/>
+      <c r="J61" s="11"/>
+      <c r="L61" s="3"/>
+      <c r="M61" s="3"/>
+      <c r="N61" s="3"/>
+      <c r="O61" s="3"/>
+    </row>
+    <row r="62" spans="4:15" x14ac:dyDescent="0.3">
+      <c r="L62" s="3"/>
+      <c r="M62" s="3"/>
+      <c r="N62" s="3"/>
+      <c r="O62" s="3"/>
+    </row>
+    <row r="63" spans="4:15" x14ac:dyDescent="0.3">
+      <c r="L63" s="3"/>
+      <c r="M63" s="3"/>
+      <c r="N63" s="3"/>
+      <c r="O63" s="3"/>
+    </row>
+    <row r="64" spans="4:15" x14ac:dyDescent="0.3">
+      <c r="L64" s="3"/>
+      <c r="M64" s="3"/>
+      <c r="N64" s="3"/>
+      <c r="O64" s="3"/>
     </row>
     <row r="65" spans="8:15" x14ac:dyDescent="0.3">
-      <c r="L65" s="4"/>
-      <c r="M65" s="4"/>
-      <c r="N65" s="4"/>
-      <c r="O65" s="4"/>
+      <c r="L65" s="3"/>
+      <c r="M65" s="3"/>
+      <c r="N65" s="3"/>
+      <c r="O65" s="3"/>
     </row>
     <row r="66" spans="8:15" x14ac:dyDescent="0.3">
-      <c r="L66" s="4"/>
-      <c r="M66" s="4"/>
-      <c r="N66" s="4"/>
-      <c r="O66" s="4"/>
+      <c r="L66" s="3"/>
+      <c r="M66" s="3"/>
+      <c r="N66" s="3"/>
+      <c r="O66" s="3"/>
     </row>
     <row r="67" spans="8:15" x14ac:dyDescent="0.3">
-      <c r="L67" s="4"/>
-      <c r="M67" s="4"/>
-      <c r="N67" s="4"/>
-      <c r="O67" s="4"/>
+      <c r="L67" s="3"/>
+      <c r="M67" s="3"/>
+      <c r="N67" s="3"/>
+      <c r="O67" s="3"/>
     </row>
     <row r="68" spans="8:15" x14ac:dyDescent="0.3">
-      <c r="L68" s="4"/>
-      <c r="M68" s="4"/>
-      <c r="N68" s="4"/>
-      <c r="O68" s="4"/>
+      <c r="L68" s="3"/>
+      <c r="M68" s="3"/>
+      <c r="N68" s="3"/>
+      <c r="O68" s="3"/>
     </row>
     <row r="69" spans="8:15" x14ac:dyDescent="0.3">
-      <c r="L69" s="4"/>
-      <c r="M69" s="4"/>
-      <c r="N69" s="4"/>
-      <c r="O69" s="4"/>
+      <c r="L69" s="3"/>
+      <c r="M69" s="3"/>
+      <c r="N69" s="3"/>
+      <c r="O69" s="3"/>
     </row>
     <row r="70" spans="8:15" x14ac:dyDescent="0.3">
-      <c r="L70" s="4"/>
-      <c r="M70" s="4"/>
-      <c r="N70" s="4"/>
-      <c r="O70" s="4"/>
+      <c r="L70" s="3"/>
+      <c r="M70" s="3"/>
+      <c r="N70" s="3"/>
+      <c r="O70" s="3"/>
     </row>
     <row r="71" spans="8:15" x14ac:dyDescent="0.3">
-      <c r="L71" s="4"/>
-      <c r="M71" s="4"/>
-      <c r="N71" s="4"/>
-      <c r="O71" s="4"/>
+      <c r="L71" s="3"/>
+      <c r="M71" s="3"/>
+      <c r="N71" s="3"/>
+      <c r="O71" s="3"/>
     </row>
     <row r="72" spans="8:15" x14ac:dyDescent="0.3">
-      <c r="L72" s="4"/>
-      <c r="M72" s="4"/>
-      <c r="N72" s="4"/>
-      <c r="O72" s="4"/>
+      <c r="L72" s="3"/>
+      <c r="M72" s="3"/>
+      <c r="N72" s="3"/>
+      <c r="O72" s="3"/>
     </row>
     <row r="73" spans="8:15" x14ac:dyDescent="0.3">
-      <c r="L73" s="4"/>
-      <c r="M73" s="4"/>
-      <c r="N73" s="4"/>
-      <c r="O73" s="4"/>
+      <c r="L73" s="3"/>
+      <c r="M73" s="3"/>
+      <c r="N73" s="3"/>
+      <c r="O73" s="3"/>
     </row>
     <row r="74" spans="8:15" x14ac:dyDescent="0.3">
-      <c r="L74" s="4"/>
-      <c r="M74" s="4"/>
-      <c r="N74" s="4"/>
-      <c r="O74" s="4"/>
+      <c r="L74" s="3"/>
+      <c r="M74" s="3"/>
+      <c r="N74" s="3"/>
+      <c r="O74" s="3"/>
     </row>
     <row r="75" spans="8:15" x14ac:dyDescent="0.3">
-      <c r="L75" s="4"/>
-      <c r="M75" s="4"/>
-      <c r="N75" s="4"/>
-      <c r="O75" s="4"/>
+      <c r="L75" s="3"/>
+      <c r="M75" s="3"/>
+      <c r="N75" s="3"/>
+      <c r="O75" s="3"/>
     </row>
     <row r="76" spans="8:15" x14ac:dyDescent="0.3">
-      <c r="L76" s="4"/>
-      <c r="M76" s="4"/>
-      <c r="N76" s="4"/>
-      <c r="O76" s="4"/>
+      <c r="L76" s="3"/>
+      <c r="M76" s="3"/>
+      <c r="N76" s="3"/>
+      <c r="O76" s="3"/>
     </row>
     <row r="78" spans="8:15" x14ac:dyDescent="0.3">
-      <c r="H78" s="4"/>
-      <c r="I78" s="4"/>
-      <c r="J78" s="4"/>
+      <c r="H78" s="3"/>
+      <c r="I78" s="3"/>
+      <c r="J78" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="57" fitToHeight="72" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="55" fitToHeight="72" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;LUBA Test Report&amp;R&amp;D</oddHeader>
     <oddFooter>Page &amp;P of &amp;N</oddFooter>
@@ -6802,25 +6996,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="9" t="s">
         <v>23</v>
       </c>
       <c r="B1" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="9" t="s">
         <v>22</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="9" t="s">
         <v>24</v>
       </c>
       <c r="F1" t="s">
         <v>26</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="9" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>